<commit_message>
AVeRA 1.0.22: in-app updater, holiday reasons, release script
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SF2.xlsx
+++ b/SF2.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://r9deped-my.sharepoint.com/personal/bonnervin_lugatiman001_r9_deped_gov_ph/Documents/WEB APP 2026/Grade Portal/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://r9deped-my.sharepoint.com/personal/bonnervin_lugatiman001_r9_deped_gov_ph/Documents/WEB APP 2026/Grade Portal EXE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{5CCDEC47-B40D-4F30-AB68-76C923403344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F25E8BF0-B204-49C7-9ACC-B4039BE0EB84}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{5CCDEC47-B40D-4F30-AB68-76C923403344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47D640B4-31B0-4C9C-89E6-838A2DA7C35E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="13896" xr2:uid="{CD8C15F5-111F-4400-810E-E3EEE55175C0}"/>
   </bookViews>
   <sheets>
     <sheet name="OCT 2026" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'OCT 2026'!$A$1:$AM$148</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1845,25 +1848,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1885,24 +1869,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1923,6 +1902,31 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1980,6 +1984,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2072,9 +2078,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2588,10 +2591,11 @@
     <col min="37" max="37" width="6.77734375" customWidth="1"/>
     <col min="38" max="38" width="7" customWidth="1"/>
     <col min="39" max="39" width="6.5546875" customWidth="1"/>
-    <col min="40" max="40" width="4.77734375" customWidth="1"/>
-    <col min="41" max="41" width="8.77734375" customWidth="1"/>
-    <col min="42" max="42" width="4.44140625" customWidth="1"/>
-    <col min="43" max="46" width="10.21875" customWidth="1"/>
+    <col min="40" max="40" width="127" hidden="1" customWidth="1"/>
+    <col min="41" max="41" width="8.77734375" hidden="1" customWidth="1"/>
+    <col min="42" max="42" width="4.44140625" hidden="1" customWidth="1"/>
+    <col min="43" max="46" width="10.21875" hidden="1" customWidth="1"/>
+    <col min="47" max="51" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:46" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2643,47 +2647,47 @@
       <c r="AT1" s="5"/>
     </row>
     <row r="2" spans="1:46" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="123" t="s">
+      <c r="A2" s="156" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="124"/>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="124"/>
-      <c r="I2" s="124"/>
-      <c r="J2" s="124"/>
-      <c r="K2" s="124"/>
-      <c r="L2" s="124"/>
-      <c r="M2" s="124"/>
-      <c r="N2" s="124"/>
-      <c r="O2" s="124"/>
-      <c r="P2" s="124"/>
-      <c r="Q2" s="124"/>
-      <c r="R2" s="124"/>
-      <c r="S2" s="124"/>
-      <c r="T2" s="124"/>
-      <c r="U2" s="124"/>
-      <c r="V2" s="124"/>
-      <c r="W2" s="124"/>
-      <c r="X2" s="124"/>
-      <c r="Y2" s="124"/>
-      <c r="Z2" s="124"/>
-      <c r="AA2" s="124"/>
-      <c r="AB2" s="124"/>
-      <c r="AC2" s="124"/>
-      <c r="AD2" s="124"/>
-      <c r="AE2" s="124"/>
-      <c r="AF2" s="124"/>
-      <c r="AG2" s="124"/>
-      <c r="AH2" s="124"/>
-      <c r="AI2" s="124"/>
-      <c r="AJ2" s="124"/>
-      <c r="AK2" s="124"/>
-      <c r="AL2" s="124"/>
-      <c r="AM2" s="124"/>
+      <c r="B2" s="134"/>
+      <c r="C2" s="134"/>
+      <c r="D2" s="134"/>
+      <c r="E2" s="134"/>
+      <c r="F2" s="134"/>
+      <c r="G2" s="134"/>
+      <c r="H2" s="134"/>
+      <c r="I2" s="134"/>
+      <c r="J2" s="134"/>
+      <c r="K2" s="134"/>
+      <c r="L2" s="134"/>
+      <c r="M2" s="134"/>
+      <c r="N2" s="134"/>
+      <c r="O2" s="134"/>
+      <c r="P2" s="134"/>
+      <c r="Q2" s="134"/>
+      <c r="R2" s="134"/>
+      <c r="S2" s="134"/>
+      <c r="T2" s="134"/>
+      <c r="U2" s="134"/>
+      <c r="V2" s="134"/>
+      <c r="W2" s="134"/>
+      <c r="X2" s="134"/>
+      <c r="Y2" s="134"/>
+      <c r="Z2" s="134"/>
+      <c r="AA2" s="134"/>
+      <c r="AB2" s="134"/>
+      <c r="AC2" s="134"/>
+      <c r="AD2" s="134"/>
+      <c r="AE2" s="134"/>
+      <c r="AF2" s="134"/>
+      <c r="AG2" s="134"/>
+      <c r="AH2" s="134"/>
+      <c r="AI2" s="134"/>
+      <c r="AJ2" s="134"/>
+      <c r="AK2" s="134"/>
+      <c r="AL2" s="134"/>
+      <c r="AM2" s="134"/>
       <c r="AN2" s="5"/>
       <c r="AO2" s="5"/>
       <c r="AP2" s="5"/>
@@ -2693,47 +2697,47 @@
       <c r="AT2" s="5"/>
     </row>
     <row r="3" spans="1:46" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="125" t="s">
+      <c r="A3" s="157" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="124"/>
-      <c r="C3" s="124"/>
-      <c r="D3" s="124"/>
-      <c r="E3" s="124"/>
-      <c r="F3" s="124"/>
-      <c r="G3" s="124"/>
-      <c r="H3" s="124"/>
-      <c r="I3" s="124"/>
-      <c r="J3" s="124"/>
-      <c r="K3" s="124"/>
-      <c r="L3" s="124"/>
-      <c r="M3" s="124"/>
-      <c r="N3" s="124"/>
-      <c r="O3" s="124"/>
-      <c r="P3" s="124"/>
-      <c r="Q3" s="124"/>
-      <c r="R3" s="124"/>
-      <c r="S3" s="124"/>
-      <c r="T3" s="124"/>
-      <c r="U3" s="124"/>
-      <c r="V3" s="124"/>
-      <c r="W3" s="124"/>
-      <c r="X3" s="124"/>
-      <c r="Y3" s="124"/>
-      <c r="Z3" s="124"/>
-      <c r="AA3" s="124"/>
-      <c r="AB3" s="124"/>
-      <c r="AC3" s="124"/>
-      <c r="AD3" s="124"/>
-      <c r="AE3" s="124"/>
-      <c r="AF3" s="124"/>
-      <c r="AG3" s="124"/>
-      <c r="AH3" s="124"/>
-      <c r="AI3" s="124"/>
-      <c r="AJ3" s="124"/>
-      <c r="AK3" s="124"/>
-      <c r="AL3" s="124"/>
-      <c r="AM3" s="124"/>
+      <c r="B3" s="134"/>
+      <c r="C3" s="134"/>
+      <c r="D3" s="134"/>
+      <c r="E3" s="134"/>
+      <c r="F3" s="134"/>
+      <c r="G3" s="134"/>
+      <c r="H3" s="134"/>
+      <c r="I3" s="134"/>
+      <c r="J3" s="134"/>
+      <c r="K3" s="134"/>
+      <c r="L3" s="134"/>
+      <c r="M3" s="134"/>
+      <c r="N3" s="134"/>
+      <c r="O3" s="134"/>
+      <c r="P3" s="134"/>
+      <c r="Q3" s="134"/>
+      <c r="R3" s="134"/>
+      <c r="S3" s="134"/>
+      <c r="T3" s="134"/>
+      <c r="U3" s="134"/>
+      <c r="V3" s="134"/>
+      <c r="W3" s="134"/>
+      <c r="X3" s="134"/>
+      <c r="Y3" s="134"/>
+      <c r="Z3" s="134"/>
+      <c r="AA3" s="134"/>
+      <c r="AB3" s="134"/>
+      <c r="AC3" s="134"/>
+      <c r="AD3" s="134"/>
+      <c r="AE3" s="134"/>
+      <c r="AF3" s="134"/>
+      <c r="AG3" s="134"/>
+      <c r="AH3" s="134"/>
+      <c r="AI3" s="134"/>
+      <c r="AJ3" s="134"/>
+      <c r="AK3" s="134"/>
+      <c r="AL3" s="134"/>
+      <c r="AM3" s="134"/>
       <c r="AN3" s="5"/>
       <c r="AO3" s="5"/>
       <c r="AP3" s="5"/>
@@ -2847,42 +2851,42 @@
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="126" t="s">
+      <c r="G6" s="135" t="s">
         <v>105</v>
       </c>
-      <c r="H6" s="127"/>
-      <c r="I6" s="127"/>
-      <c r="J6" s="128"/>
+      <c r="H6" s="136"/>
+      <c r="I6" s="136"/>
+      <c r="J6" s="137"/>
       <c r="K6" s="8"/>
       <c r="L6" s="8"/>
       <c r="M6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="N6" s="126" t="s">
+      <c r="N6" s="135" t="s">
         <v>102</v>
       </c>
-      <c r="O6" s="127"/>
-      <c r="P6" s="127"/>
-      <c r="Q6" s="127"/>
-      <c r="R6" s="128"/>
+      <c r="O6" s="136"/>
+      <c r="P6" s="136"/>
+      <c r="Q6" s="136"/>
+      <c r="R6" s="137"/>
       <c r="S6" s="8"/>
-      <c r="T6" s="129" t="s">
+      <c r="T6" s="138" t="s">
         <v>4</v>
       </c>
-      <c r="U6" s="124"/>
-      <c r="V6" s="124"/>
-      <c r="W6" s="124"/>
-      <c r="X6" s="124"/>
-      <c r="Y6" s="124"/>
-      <c r="Z6" s="130"/>
-      <c r="AA6" s="131" t="s">
+      <c r="U6" s="134"/>
+      <c r="V6" s="134"/>
+      <c r="W6" s="134"/>
+      <c r="X6" s="134"/>
+      <c r="Y6" s="134"/>
+      <c r="Z6" s="139"/>
+      <c r="AA6" s="158" t="s">
         <v>101</v>
       </c>
-      <c r="AB6" s="127"/>
-      <c r="AC6" s="127"/>
-      <c r="AD6" s="127"/>
-      <c r="AE6" s="127"/>
-      <c r="AF6" s="128"/>
+      <c r="AB6" s="136"/>
+      <c r="AC6" s="136"/>
+      <c r="AD6" s="136"/>
+      <c r="AE6" s="136"/>
+      <c r="AF6" s="137"/>
       <c r="AG6" s="8"/>
       <c r="AH6" s="8"/>
       <c r="AI6" s="8"/>
@@ -2891,14 +2895,14 @@
       <c r="AL6" s="6"/>
       <c r="AM6" s="6"/>
       <c r="AN6" s="5"/>
-      <c r="AO6" s="142" t="s">
+      <c r="AO6" s="133" t="s">
         <v>5</v>
       </c>
-      <c r="AP6" s="124"/>
-      <c r="AQ6" s="124"/>
-      <c r="AR6" s="124"/>
-      <c r="AS6" s="124"/>
-      <c r="AT6" s="124"/>
+      <c r="AP6" s="134"/>
+      <c r="AQ6" s="134"/>
+      <c r="AR6" s="134"/>
+      <c r="AS6" s="134"/>
+      <c r="AT6" s="134"/>
     </row>
     <row r="7" spans="1:46" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
@@ -2909,47 +2913,47 @@
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
-      <c r="G7" s="126" t="s">
+      <c r="G7" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="127"/>
-      <c r="I7" s="127"/>
-      <c r="J7" s="127"/>
-      <c r="K7" s="127"/>
-      <c r="L7" s="127"/>
-      <c r="M7" s="127"/>
-      <c r="N7" s="127"/>
-      <c r="O7" s="127"/>
-      <c r="P7" s="127"/>
-      <c r="Q7" s="127"/>
-      <c r="R7" s="128"/>
+      <c r="H7" s="136"/>
+      <c r="I7" s="136"/>
+      <c r="J7" s="136"/>
+      <c r="K7" s="136"/>
+      <c r="L7" s="136"/>
+      <c r="M7" s="136"/>
+      <c r="N7" s="136"/>
+      <c r="O7" s="136"/>
+      <c r="P7" s="136"/>
+      <c r="Q7" s="136"/>
+      <c r="R7" s="137"/>
       <c r="S7" s="11"/>
       <c r="T7" s="11"/>
       <c r="U7" s="11"/>
       <c r="V7" s="11"/>
-      <c r="W7" s="129" t="s">
+      <c r="W7" s="138" t="s">
         <v>7</v>
       </c>
-      <c r="X7" s="124"/>
-      <c r="Y7" s="124"/>
-      <c r="Z7" s="130"/>
-      <c r="AA7" s="126" t="s">
+      <c r="X7" s="134"/>
+      <c r="Y7" s="134"/>
+      <c r="Z7" s="139"/>
+      <c r="AA7" s="135" t="s">
         <v>104</v>
       </c>
-      <c r="AB7" s="128"/>
-      <c r="AC7" s="143" t="s">
+      <c r="AB7" s="137"/>
+      <c r="AC7" s="140" t="s">
         <v>8</v>
       </c>
-      <c r="AD7" s="124"/>
-      <c r="AE7" s="130"/>
-      <c r="AF7" s="126" t="s">
+      <c r="AD7" s="134"/>
+      <c r="AE7" s="139"/>
+      <c r="AF7" s="135" t="s">
         <v>103</v>
       </c>
-      <c r="AG7" s="127"/>
-      <c r="AH7" s="127"/>
-      <c r="AI7" s="127"/>
-      <c r="AJ7" s="127"/>
-      <c r="AK7" s="128"/>
+      <c r="AG7" s="136"/>
+      <c r="AH7" s="136"/>
+      <c r="AI7" s="136"/>
+      <c r="AJ7" s="136"/>
+      <c r="AK7" s="137"/>
       <c r="AL7" s="10"/>
       <c r="AM7" s="10"/>
       <c r="AN7" s="5"/>
@@ -3009,59 +3013,59 @@
       <c r="AT8" s="5"/>
     </row>
     <row r="9" spans="1:46" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="151" t="s">
+      <c r="A9" s="141" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="152"/>
+      <c r="B9" s="142"/>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
-      <c r="G9" s="154" t="s">
+      <c r="G9" s="144" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="155"/>
-      <c r="I9" s="155"/>
-      <c r="J9" s="155"/>
-      <c r="K9" s="155"/>
-      <c r="L9" s="155"/>
-      <c r="M9" s="155"/>
-      <c r="N9" s="155"/>
-      <c r="O9" s="155"/>
-      <c r="P9" s="155"/>
-      <c r="Q9" s="155"/>
-      <c r="R9" s="155"/>
-      <c r="S9" s="155"/>
-      <c r="T9" s="155"/>
-      <c r="U9" s="155"/>
-      <c r="V9" s="155"/>
-      <c r="W9" s="155"/>
-      <c r="X9" s="155"/>
-      <c r="Y9" s="155"/>
-      <c r="Z9" s="155"/>
-      <c r="AA9" s="155"/>
-      <c r="AB9" s="155"/>
-      <c r="AC9" s="155"/>
-      <c r="AD9" s="155"/>
-      <c r="AE9" s="156"/>
-      <c r="AF9" s="157" t="s">
+      <c r="H9" s="145"/>
+      <c r="I9" s="145"/>
+      <c r="J9" s="145"/>
+      <c r="K9" s="145"/>
+      <c r="L9" s="145"/>
+      <c r="M9" s="145"/>
+      <c r="N9" s="145"/>
+      <c r="O9" s="145"/>
+      <c r="P9" s="145"/>
+      <c r="Q9" s="145"/>
+      <c r="R9" s="145"/>
+      <c r="S9" s="145"/>
+      <c r="T9" s="145"/>
+      <c r="U9" s="145"/>
+      <c r="V9" s="145"/>
+      <c r="W9" s="145"/>
+      <c r="X9" s="145"/>
+      <c r="Y9" s="145"/>
+      <c r="Z9" s="145"/>
+      <c r="AA9" s="145"/>
+      <c r="AB9" s="145"/>
+      <c r="AC9" s="145"/>
+      <c r="AD9" s="145"/>
+      <c r="AE9" s="146"/>
+      <c r="AF9" s="147" t="s">
         <v>11</v>
       </c>
-      <c r="AG9" s="152"/>
-      <c r="AH9" s="159" t="s">
+      <c r="AG9" s="142"/>
+      <c r="AH9" s="149" t="s">
         <v>12</v>
       </c>
-      <c r="AI9" s="152"/>
-      <c r="AJ9" s="152"/>
-      <c r="AK9" s="152"/>
-      <c r="AL9" s="152"/>
-      <c r="AM9" s="160"/>
+      <c r="AI9" s="142"/>
+      <c r="AJ9" s="142"/>
+      <c r="AK9" s="142"/>
+      <c r="AL9" s="142"/>
+      <c r="AM9" s="150"/>
       <c r="AN9" s="5"/>
-      <c r="AO9" s="132" t="s">
+      <c r="AO9" s="123" t="s">
         <v>13</v>
       </c>
-      <c r="AP9" s="133"/>
-      <c r="AQ9" s="136">
+      <c r="AP9" s="124"/>
+      <c r="AQ9" s="127">
         <v>16</v>
       </c>
       <c r="AR9" s="5"/>
@@ -3069,8 +3073,8 @@
       <c r="AT9" s="5"/>
     </row>
     <row r="10" spans="1:46" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="153"/>
-      <c r="B10" s="124"/>
+      <c r="A10" s="143"/>
+      <c r="B10" s="134"/>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
@@ -3144,25 +3148,25 @@
       <c r="AE10" s="17">
         <v>30</v>
       </c>
-      <c r="AF10" s="158"/>
-      <c r="AG10" s="158"/>
-      <c r="AH10" s="153"/>
-      <c r="AI10" s="124"/>
-      <c r="AJ10" s="124"/>
-      <c r="AK10" s="124"/>
-      <c r="AL10" s="124"/>
-      <c r="AM10" s="161"/>
+      <c r="AF10" s="148"/>
+      <c r="AG10" s="148"/>
+      <c r="AH10" s="143"/>
+      <c r="AI10" s="134"/>
+      <c r="AJ10" s="134"/>
+      <c r="AK10" s="134"/>
+      <c r="AL10" s="134"/>
+      <c r="AM10" s="151"/>
       <c r="AN10" s="5"/>
-      <c r="AO10" s="134"/>
-      <c r="AP10" s="135"/>
-      <c r="AQ10" s="137"/>
+      <c r="AO10" s="125"/>
+      <c r="AP10" s="126"/>
+      <c r="AQ10" s="128"/>
       <c r="AR10" s="5"/>
       <c r="AS10" s="5"/>
       <c r="AT10" s="5"/>
     </row>
     <row r="11" spans="1:46" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="153"/>
-      <c r="B11" s="124"/>
+      <c r="A11" s="143"/>
+      <c r="B11" s="134"/>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
@@ -3242,18 +3246,18 @@
       <c r="AE11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="AF11" s="138" t="s">
+      <c r="AF11" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="AG11" s="140" t="s">
+      <c r="AG11" s="131" t="s">
         <v>20</v>
       </c>
-      <c r="AH11" s="153"/>
-      <c r="AI11" s="124"/>
-      <c r="AJ11" s="124"/>
-      <c r="AK11" s="124"/>
-      <c r="AL11" s="124"/>
-      <c r="AM11" s="161"/>
+      <c r="AH11" s="143"/>
+      <c r="AI11" s="134"/>
+      <c r="AJ11" s="134"/>
+      <c r="AK11" s="134"/>
+      <c r="AL11" s="134"/>
+      <c r="AM11" s="151"/>
       <c r="AN11" s="5"/>
       <c r="AO11" s="5"/>
       <c r="AP11" s="5"/>
@@ -3296,14 +3300,14 @@
       <c r="AC12" s="28"/>
       <c r="AD12" s="31"/>
       <c r="AE12" s="29"/>
-      <c r="AF12" s="139"/>
-      <c r="AG12" s="141"/>
-      <c r="AH12" s="162"/>
-      <c r="AI12" s="158"/>
-      <c r="AJ12" s="158"/>
-      <c r="AK12" s="158"/>
-      <c r="AL12" s="158"/>
-      <c r="AM12" s="139"/>
+      <c r="AF12" s="130"/>
+      <c r="AG12" s="132"/>
+      <c r="AH12" s="152"/>
+      <c r="AI12" s="148"/>
+      <c r="AJ12" s="148"/>
+      <c r="AK12" s="148"/>
+      <c r="AL12" s="148"/>
+      <c r="AM12" s="130"/>
       <c r="AN12" s="5"/>
       <c r="AO12" s="5"/>
       <c r="AP12" s="5"/>
@@ -3354,12 +3358,12 @@
         <f t="shared" ref="AG13:AG62" si="1">IF(B13="","",$AJ$117-AF13)</f>
         <v/>
       </c>
-      <c r="AH13" s="144"/>
-      <c r="AI13" s="146"/>
-      <c r="AJ13" s="146"/>
-      <c r="AK13" s="146"/>
-      <c r="AL13" s="146"/>
-      <c r="AM13" s="221"/>
+      <c r="AH13" s="153"/>
+      <c r="AI13" s="154"/>
+      <c r="AJ13" s="154"/>
+      <c r="AK13" s="154"/>
+      <c r="AL13" s="154"/>
+      <c r="AM13" s="155"/>
       <c r="AN13" s="5"/>
       <c r="AO13" s="2" t="s">
         <v>23</v>
@@ -3412,12 +3416,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH14" s="144"/>
-      <c r="AI14" s="146"/>
-      <c r="AJ14" s="146"/>
-      <c r="AK14" s="146"/>
-      <c r="AL14" s="146"/>
-      <c r="AM14" s="221"/>
+      <c r="AH14" s="153"/>
+      <c r="AI14" s="154"/>
+      <c r="AJ14" s="154"/>
+      <c r="AK14" s="154"/>
+      <c r="AL14" s="154"/>
+      <c r="AM14" s="155"/>
       <c r="AN14" s="5"/>
       <c r="AO14" s="9" t="s">
         <v>24</v>
@@ -3472,12 +3476,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH15" s="144"/>
-      <c r="AI15" s="146"/>
-      <c r="AJ15" s="146"/>
-      <c r="AK15" s="146"/>
-      <c r="AL15" s="146"/>
-      <c r="AM15" s="221"/>
+      <c r="AH15" s="153"/>
+      <c r="AI15" s="154"/>
+      <c r="AJ15" s="154"/>
+      <c r="AK15" s="154"/>
+      <c r="AL15" s="154"/>
+      <c r="AM15" s="155"/>
       <c r="AN15" s="5"/>
       <c r="AO15" s="9" t="s">
         <v>22</v>
@@ -3532,12 +3536,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH16" s="144"/>
-      <c r="AI16" s="146"/>
-      <c r="AJ16" s="146"/>
-      <c r="AK16" s="146"/>
-      <c r="AL16" s="146"/>
-      <c r="AM16" s="221"/>
+      <c r="AH16" s="153"/>
+      <c r="AI16" s="154"/>
+      <c r="AJ16" s="154"/>
+      <c r="AK16" s="154"/>
+      <c r="AL16" s="154"/>
+      <c r="AM16" s="155"/>
       <c r="AN16" s="5"/>
       <c r="AO16" s="9" t="s">
         <v>26</v>
@@ -3592,12 +3596,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH17" s="144"/>
-      <c r="AI17" s="146"/>
-      <c r="AJ17" s="146"/>
-      <c r="AK17" s="146"/>
-      <c r="AL17" s="146"/>
-      <c r="AM17" s="221"/>
+      <c r="AH17" s="153"/>
+      <c r="AI17" s="154"/>
+      <c r="AJ17" s="154"/>
+      <c r="AK17" s="154"/>
+      <c r="AL17" s="154"/>
+      <c r="AM17" s="155"/>
       <c r="AN17" s="5"/>
       <c r="AO17" s="5"/>
       <c r="AP17" s="5"/>
@@ -3648,12 +3652,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH18" s="144"/>
-      <c r="AI18" s="146"/>
-      <c r="AJ18" s="146"/>
-      <c r="AK18" s="146"/>
-      <c r="AL18" s="146"/>
-      <c r="AM18" s="221"/>
+      <c r="AH18" s="153"/>
+      <c r="AI18" s="154"/>
+      <c r="AJ18" s="154"/>
+      <c r="AK18" s="154"/>
+      <c r="AL18" s="154"/>
+      <c r="AM18" s="155"/>
       <c r="AN18" s="5"/>
       <c r="AO18" s="2" t="s">
         <v>29</v>
@@ -3708,12 +3712,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH19" s="144"/>
-      <c r="AI19" s="146"/>
-      <c r="AJ19" s="146"/>
-      <c r="AK19" s="146"/>
-      <c r="AL19" s="146"/>
-      <c r="AM19" s="221"/>
+      <c r="AH19" s="153"/>
+      <c r="AI19" s="154"/>
+      <c r="AJ19" s="154"/>
+      <c r="AK19" s="154"/>
+      <c r="AL19" s="154"/>
+      <c r="AM19" s="155"/>
       <c r="AN19" s="5"/>
       <c r="AO19" s="5"/>
       <c r="AP19" s="5"/>
@@ -3764,12 +3768,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH20" s="144"/>
-      <c r="AI20" s="146"/>
-      <c r="AJ20" s="146"/>
-      <c r="AK20" s="146"/>
-      <c r="AL20" s="146"/>
-      <c r="AM20" s="221"/>
+      <c r="AH20" s="153"/>
+      <c r="AI20" s="154"/>
+      <c r="AJ20" s="154"/>
+      <c r="AK20" s="154"/>
+      <c r="AL20" s="154"/>
+      <c r="AM20" s="155"/>
       <c r="AN20" s="5"/>
       <c r="AO20" s="5"/>
       <c r="AP20" s="5"/>
@@ -3820,12 +3824,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH21" s="144"/>
-      <c r="AI21" s="146"/>
-      <c r="AJ21" s="146"/>
-      <c r="AK21" s="146"/>
-      <c r="AL21" s="146"/>
-      <c r="AM21" s="221"/>
+      <c r="AH21" s="153"/>
+      <c r="AI21" s="154"/>
+      <c r="AJ21" s="154"/>
+      <c r="AK21" s="154"/>
+      <c r="AL21" s="154"/>
+      <c r="AM21" s="155"/>
       <c r="AN21" s="5"/>
       <c r="AO21" s="5"/>
       <c r="AP21" s="5"/>
@@ -3876,12 +3880,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH22" s="144"/>
-      <c r="AI22" s="146"/>
-      <c r="AJ22" s="146"/>
-      <c r="AK22" s="146"/>
-      <c r="AL22" s="146"/>
-      <c r="AM22" s="221"/>
+      <c r="AH22" s="153"/>
+      <c r="AI22" s="154"/>
+      <c r="AJ22" s="154"/>
+      <c r="AK22" s="154"/>
+      <c r="AL22" s="154"/>
+      <c r="AM22" s="155"/>
       <c r="AN22" s="5"/>
       <c r="AO22" s="5"/>
       <c r="AP22" s="5"/>
@@ -3932,12 +3936,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH23" s="144"/>
-      <c r="AI23" s="146"/>
-      <c r="AJ23" s="146"/>
-      <c r="AK23" s="146"/>
-      <c r="AL23" s="146"/>
-      <c r="AM23" s="221"/>
+      <c r="AH23" s="153"/>
+      <c r="AI23" s="154"/>
+      <c r="AJ23" s="154"/>
+      <c r="AK23" s="154"/>
+      <c r="AL23" s="154"/>
+      <c r="AM23" s="155"/>
       <c r="AN23" s="5"/>
       <c r="AO23" s="5"/>
       <c r="AP23" s="5"/>
@@ -3988,12 +3992,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH24" s="148"/>
-      <c r="AI24" s="127"/>
-      <c r="AJ24" s="149"/>
-      <c r="AK24" s="127"/>
-      <c r="AL24" s="127"/>
-      <c r="AM24" s="150"/>
+      <c r="AH24" s="159"/>
+      <c r="AI24" s="136"/>
+      <c r="AJ24" s="160"/>
+      <c r="AK24" s="136"/>
+      <c r="AL24" s="136"/>
+      <c r="AM24" s="161"/>
       <c r="AN24" s="5"/>
       <c r="AO24" s="5"/>
       <c r="AP24" s="5"/>
@@ -4044,12 +4048,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH25" s="148"/>
-      <c r="AI25" s="127"/>
-      <c r="AJ25" s="149"/>
-      <c r="AK25" s="127"/>
-      <c r="AL25" s="127"/>
-      <c r="AM25" s="150"/>
+      <c r="AH25" s="159"/>
+      <c r="AI25" s="136"/>
+      <c r="AJ25" s="160"/>
+      <c r="AK25" s="136"/>
+      <c r="AL25" s="136"/>
+      <c r="AM25" s="161"/>
       <c r="AN25" s="5"/>
       <c r="AO25" s="5"/>
       <c r="AP25" s="5"/>
@@ -4100,12 +4104,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH26" s="148"/>
-      <c r="AI26" s="127"/>
-      <c r="AJ26" s="149"/>
-      <c r="AK26" s="127"/>
-      <c r="AL26" s="127"/>
-      <c r="AM26" s="150"/>
+      <c r="AH26" s="159"/>
+      <c r="AI26" s="136"/>
+      <c r="AJ26" s="160"/>
+      <c r="AK26" s="136"/>
+      <c r="AL26" s="136"/>
+      <c r="AM26" s="161"/>
       <c r="AN26" s="5"/>
       <c r="AO26" s="5"/>
       <c r="AP26" s="5"/>
@@ -4156,12 +4160,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH27" s="148"/>
-      <c r="AI27" s="127"/>
-      <c r="AJ27" s="149"/>
-      <c r="AK27" s="127"/>
-      <c r="AL27" s="127"/>
-      <c r="AM27" s="150"/>
+      <c r="AH27" s="159"/>
+      <c r="AI27" s="136"/>
+      <c r="AJ27" s="160"/>
+      <c r="AK27" s="136"/>
+      <c r="AL27" s="136"/>
+      <c r="AM27" s="161"/>
       <c r="AN27" s="5"/>
       <c r="AO27" s="5"/>
       <c r="AP27" s="5"/>
@@ -4212,12 +4216,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH28" s="148"/>
-      <c r="AI28" s="127"/>
-      <c r="AJ28" s="149"/>
-      <c r="AK28" s="127"/>
-      <c r="AL28" s="127"/>
-      <c r="AM28" s="150"/>
+      <c r="AH28" s="159"/>
+      <c r="AI28" s="136"/>
+      <c r="AJ28" s="160"/>
+      <c r="AK28" s="136"/>
+      <c r="AL28" s="136"/>
+      <c r="AM28" s="161"/>
       <c r="AN28" s="5"/>
       <c r="AO28" s="5"/>
       <c r="AP28" s="5"/>
@@ -4268,12 +4272,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH29" s="148"/>
-      <c r="AI29" s="127"/>
-      <c r="AJ29" s="149"/>
-      <c r="AK29" s="127"/>
-      <c r="AL29" s="127"/>
-      <c r="AM29" s="150"/>
+      <c r="AH29" s="159"/>
+      <c r="AI29" s="136"/>
+      <c r="AJ29" s="160"/>
+      <c r="AK29" s="136"/>
+      <c r="AL29" s="136"/>
+      <c r="AM29" s="161"/>
       <c r="AN29" s="5"/>
       <c r="AO29" s="5"/>
       <c r="AP29" s="5"/>
@@ -4324,12 +4328,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH30" s="148"/>
-      <c r="AI30" s="127"/>
-      <c r="AJ30" s="149"/>
-      <c r="AK30" s="127"/>
-      <c r="AL30" s="127"/>
-      <c r="AM30" s="150"/>
+      <c r="AH30" s="159"/>
+      <c r="AI30" s="136"/>
+      <c r="AJ30" s="160"/>
+      <c r="AK30" s="136"/>
+      <c r="AL30" s="136"/>
+      <c r="AM30" s="161"/>
       <c r="AN30" s="5"/>
       <c r="AO30" s="5"/>
       <c r="AP30" s="5"/>
@@ -4380,8 +4384,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH31" s="148"/>
-      <c r="AI31" s="127"/>
+      <c r="AH31" s="159"/>
+      <c r="AI31" s="136"/>
       <c r="AJ31" s="53"/>
       <c r="AK31" s="53"/>
       <c r="AL31" s="53"/>
@@ -4436,8 +4440,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH32" s="148"/>
-      <c r="AI32" s="127"/>
+      <c r="AH32" s="159"/>
+      <c r="AI32" s="136"/>
       <c r="AJ32" s="53"/>
       <c r="AK32" s="53"/>
       <c r="AL32" s="53"/>
@@ -4492,8 +4496,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH33" s="148"/>
-      <c r="AI33" s="127"/>
+      <c r="AH33" s="159"/>
+      <c r="AI33" s="136"/>
       <c r="AJ33" s="53"/>
       <c r="AK33" s="53"/>
       <c r="AL33" s="53"/>
@@ -4548,8 +4552,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH34" s="148"/>
-      <c r="AI34" s="127"/>
+      <c r="AH34" s="159"/>
+      <c r="AI34" s="136"/>
       <c r="AJ34" s="53"/>
       <c r="AK34" s="53"/>
       <c r="AL34" s="53"/>
@@ -4604,8 +4608,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH35" s="148"/>
-      <c r="AI35" s="127"/>
+      <c r="AH35" s="159"/>
+      <c r="AI35" s="136"/>
       <c r="AJ35" s="53"/>
       <c r="AK35" s="53"/>
       <c r="AL35" s="53"/>
@@ -4660,8 +4664,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH36" s="148"/>
-      <c r="AI36" s="127"/>
+      <c r="AH36" s="159"/>
+      <c r="AI36" s="136"/>
       <c r="AJ36" s="53"/>
       <c r="AK36" s="53"/>
       <c r="AL36" s="53"/>
@@ -4716,8 +4720,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH37" s="148"/>
-      <c r="AI37" s="127"/>
+      <c r="AH37" s="159"/>
+      <c r="AI37" s="136"/>
       <c r="AJ37" s="53"/>
       <c r="AK37" s="53"/>
       <c r="AL37" s="53"/>
@@ -4772,8 +4776,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH38" s="148"/>
-      <c r="AI38" s="127"/>
+      <c r="AH38" s="159"/>
+      <c r="AI38" s="136"/>
       <c r="AJ38" s="53"/>
       <c r="AK38" s="53"/>
       <c r="AL38" s="53"/>
@@ -4828,8 +4832,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH39" s="148"/>
-      <c r="AI39" s="127"/>
+      <c r="AH39" s="159"/>
+      <c r="AI39" s="136"/>
       <c r="AJ39" s="53"/>
       <c r="AK39" s="53"/>
       <c r="AL39" s="53"/>
@@ -4884,8 +4888,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH40" s="148"/>
-      <c r="AI40" s="127"/>
+      <c r="AH40" s="159"/>
+      <c r="AI40" s="136"/>
       <c r="AJ40" s="53"/>
       <c r="AK40" s="53"/>
       <c r="AL40" s="53"/>
@@ -4940,8 +4944,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH41" s="148"/>
-      <c r="AI41" s="127"/>
+      <c r="AH41" s="159"/>
+      <c r="AI41" s="136"/>
       <c r="AJ41" s="53"/>
       <c r="AK41" s="53"/>
       <c r="AL41" s="53"/>
@@ -4996,12 +5000,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH42" s="148"/>
-      <c r="AI42" s="127"/>
-      <c r="AJ42" s="149"/>
-      <c r="AK42" s="127"/>
-      <c r="AL42" s="127"/>
-      <c r="AM42" s="150"/>
+      <c r="AH42" s="159"/>
+      <c r="AI42" s="136"/>
+      <c r="AJ42" s="160"/>
+      <c r="AK42" s="136"/>
+      <c r="AL42" s="136"/>
+      <c r="AM42" s="161"/>
       <c r="AN42" s="5"/>
       <c r="AO42" s="5"/>
       <c r="AP42" s="5"/>
@@ -5052,8 +5056,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH43" s="148"/>
-      <c r="AI43" s="127"/>
+      <c r="AH43" s="159"/>
+      <c r="AI43" s="136"/>
       <c r="AJ43" s="53"/>
       <c r="AK43" s="53"/>
       <c r="AL43" s="53"/>
@@ -5108,8 +5112,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH44" s="148"/>
-      <c r="AI44" s="127"/>
+      <c r="AH44" s="159"/>
+      <c r="AI44" s="136"/>
       <c r="AJ44" s="53"/>
       <c r="AK44" s="53"/>
       <c r="AL44" s="53"/>
@@ -5164,8 +5168,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH45" s="148"/>
-      <c r="AI45" s="127"/>
+      <c r="AH45" s="159"/>
+      <c r="AI45" s="136"/>
       <c r="AJ45" s="53"/>
       <c r="AK45" s="53"/>
       <c r="AL45" s="53"/>
@@ -5220,8 +5224,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH46" s="148"/>
-      <c r="AI46" s="127"/>
+      <c r="AH46" s="159"/>
+      <c r="AI46" s="136"/>
       <c r="AJ46" s="53"/>
       <c r="AK46" s="53"/>
       <c r="AL46" s="53"/>
@@ -5276,8 +5280,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH47" s="148"/>
-      <c r="AI47" s="127"/>
+      <c r="AH47" s="159"/>
+      <c r="AI47" s="136"/>
       <c r="AJ47" s="53"/>
       <c r="AK47" s="53"/>
       <c r="AL47" s="53"/>
@@ -5332,8 +5336,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH48" s="148"/>
-      <c r="AI48" s="127"/>
+      <c r="AH48" s="159"/>
+      <c r="AI48" s="136"/>
       <c r="AJ48" s="53"/>
       <c r="AK48" s="53"/>
       <c r="AL48" s="53"/>
@@ -5388,8 +5392,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH49" s="148"/>
-      <c r="AI49" s="127"/>
+      <c r="AH49" s="159"/>
+      <c r="AI49" s="136"/>
       <c r="AJ49" s="53"/>
       <c r="AK49" s="53"/>
       <c r="AL49" s="53"/>
@@ -5444,8 +5448,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH50" s="148"/>
-      <c r="AI50" s="127"/>
+      <c r="AH50" s="159"/>
+      <c r="AI50" s="136"/>
       <c r="AJ50" s="53"/>
       <c r="AK50" s="53"/>
       <c r="AL50" s="53"/>
@@ -5500,8 +5504,8 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH51" s="148"/>
-      <c r="AI51" s="127"/>
+      <c r="AH51" s="159"/>
+      <c r="AI51" s="136"/>
       <c r="AJ51" s="53"/>
       <c r="AK51" s="53"/>
       <c r="AL51" s="53"/>
@@ -5556,12 +5560,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH52" s="148"/>
-      <c r="AI52" s="127"/>
-      <c r="AJ52" s="149"/>
-      <c r="AK52" s="127"/>
-      <c r="AL52" s="127"/>
-      <c r="AM52" s="150"/>
+      <c r="AH52" s="159"/>
+      <c r="AI52" s="136"/>
+      <c r="AJ52" s="160"/>
+      <c r="AK52" s="136"/>
+      <c r="AL52" s="136"/>
+      <c r="AM52" s="161"/>
       <c r="AN52" s="5"/>
       <c r="AO52" s="5"/>
       <c r="AP52" s="5"/>
@@ -5612,12 +5616,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH53" s="148"/>
-      <c r="AI53" s="127"/>
-      <c r="AJ53" s="149"/>
-      <c r="AK53" s="127"/>
-      <c r="AL53" s="127"/>
-      <c r="AM53" s="150"/>
+      <c r="AH53" s="159"/>
+      <c r="AI53" s="136"/>
+      <c r="AJ53" s="160"/>
+      <c r="AK53" s="136"/>
+      <c r="AL53" s="136"/>
+      <c r="AM53" s="161"/>
       <c r="AN53" s="5"/>
       <c r="AO53" s="5"/>
       <c r="AP53" s="5"/>
@@ -5668,12 +5672,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH54" s="148"/>
-      <c r="AI54" s="127"/>
-      <c r="AJ54" s="149"/>
-      <c r="AK54" s="127"/>
-      <c r="AL54" s="127"/>
-      <c r="AM54" s="150"/>
+      <c r="AH54" s="159"/>
+      <c r="AI54" s="136"/>
+      <c r="AJ54" s="160"/>
+      <c r="AK54" s="136"/>
+      <c r="AL54" s="136"/>
+      <c r="AM54" s="161"/>
       <c r="AN54" s="5"/>
       <c r="AO54" s="5"/>
       <c r="AP54" s="5"/>
@@ -5724,12 +5728,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH55" s="148"/>
-      <c r="AI55" s="127"/>
-      <c r="AJ55" s="149"/>
-      <c r="AK55" s="127"/>
-      <c r="AL55" s="127"/>
-      <c r="AM55" s="150"/>
+      <c r="AH55" s="159"/>
+      <c r="AI55" s="136"/>
+      <c r="AJ55" s="160"/>
+      <c r="AK55" s="136"/>
+      <c r="AL55" s="136"/>
+      <c r="AM55" s="161"/>
       <c r="AN55" s="5"/>
       <c r="AO55" s="5"/>
       <c r="AP55" s="5"/>
@@ -5780,12 +5784,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH56" s="148"/>
-      <c r="AI56" s="127"/>
-      <c r="AJ56" s="149"/>
-      <c r="AK56" s="127"/>
-      <c r="AL56" s="127"/>
-      <c r="AM56" s="150"/>
+      <c r="AH56" s="159"/>
+      <c r="AI56" s="136"/>
+      <c r="AJ56" s="160"/>
+      <c r="AK56" s="136"/>
+      <c r="AL56" s="136"/>
+      <c r="AM56" s="161"/>
       <c r="AN56" s="5"/>
       <c r="AO56" s="5"/>
       <c r="AP56" s="5"/>
@@ -5836,12 +5840,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH57" s="148"/>
-      <c r="AI57" s="127"/>
-      <c r="AJ57" s="149"/>
-      <c r="AK57" s="127"/>
-      <c r="AL57" s="127"/>
-      <c r="AM57" s="150"/>
+      <c r="AH57" s="159"/>
+      <c r="AI57" s="136"/>
+      <c r="AJ57" s="160"/>
+      <c r="AK57" s="136"/>
+      <c r="AL57" s="136"/>
+      <c r="AM57" s="161"/>
       <c r="AN57" s="5"/>
       <c r="AO57" s="5"/>
       <c r="AP57" s="5"/>
@@ -5892,12 +5896,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH58" s="148"/>
-      <c r="AI58" s="127"/>
-      <c r="AJ58" s="149"/>
-      <c r="AK58" s="127"/>
-      <c r="AL58" s="127"/>
-      <c r="AM58" s="150"/>
+      <c r="AH58" s="159"/>
+      <c r="AI58" s="136"/>
+      <c r="AJ58" s="160"/>
+      <c r="AK58" s="136"/>
+      <c r="AL58" s="136"/>
+      <c r="AM58" s="161"/>
       <c r="AN58" s="5"/>
       <c r="AO58" s="5"/>
       <c r="AP58" s="5"/>
@@ -5948,12 +5952,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH59" s="148"/>
-      <c r="AI59" s="127"/>
-      <c r="AJ59" s="149"/>
-      <c r="AK59" s="127"/>
-      <c r="AL59" s="127"/>
-      <c r="AM59" s="150"/>
+      <c r="AH59" s="159"/>
+      <c r="AI59" s="136"/>
+      <c r="AJ59" s="160"/>
+      <c r="AK59" s="136"/>
+      <c r="AL59" s="136"/>
+      <c r="AM59" s="161"/>
       <c r="AN59" s="5"/>
       <c r="AO59" s="5"/>
       <c r="AP59" s="5"/>
@@ -6004,12 +6008,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH60" s="148"/>
-      <c r="AI60" s="127"/>
-      <c r="AJ60" s="149"/>
-      <c r="AK60" s="127"/>
-      <c r="AL60" s="127"/>
-      <c r="AM60" s="150"/>
+      <c r="AH60" s="159"/>
+      <c r="AI60" s="136"/>
+      <c r="AJ60" s="160"/>
+      <c r="AK60" s="136"/>
+      <c r="AL60" s="136"/>
+      <c r="AM60" s="161"/>
       <c r="AN60" s="5"/>
       <c r="AO60" s="5"/>
       <c r="AP60" s="5"/>
@@ -6060,12 +6064,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH61" s="148"/>
-      <c r="AI61" s="127"/>
-      <c r="AJ61" s="149"/>
-      <c r="AK61" s="127"/>
-      <c r="AL61" s="127"/>
-      <c r="AM61" s="150"/>
+      <c r="AH61" s="159"/>
+      <c r="AI61" s="136"/>
+      <c r="AJ61" s="160"/>
+      <c r="AK61" s="136"/>
+      <c r="AL61" s="136"/>
+      <c r="AM61" s="161"/>
       <c r="AN61" s="5"/>
       <c r="AO61" s="5"/>
       <c r="AP61" s="5"/>
@@ -6116,12 +6120,12 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="AH62" s="148"/>
-      <c r="AI62" s="127"/>
-      <c r="AJ62" s="163"/>
-      <c r="AK62" s="164"/>
-      <c r="AL62" s="164"/>
-      <c r="AM62" s="165"/>
+      <c r="AH62" s="159"/>
+      <c r="AI62" s="136"/>
+      <c r="AJ62" s="162"/>
+      <c r="AK62" s="163"/>
+      <c r="AL62" s="163"/>
+      <c r="AM62" s="164"/>
       <c r="AN62" s="5"/>
       <c r="AO62" s="5"/>
       <c r="AP62" s="5"/>
@@ -6303,12 +6307,12 @@
         <f t="shared" ref="AG64:AG113" si="5">IF(B64="","",$AJ$117-AF64)</f>
         <v/>
       </c>
-      <c r="AH64" s="144"/>
-      <c r="AI64" s="146"/>
-      <c r="AJ64" s="146"/>
-      <c r="AK64" s="146"/>
-      <c r="AL64" s="146"/>
-      <c r="AM64" s="221"/>
+      <c r="AH64" s="153"/>
+      <c r="AI64" s="154"/>
+      <c r="AJ64" s="154"/>
+      <c r="AK64" s="154"/>
+      <c r="AL64" s="154"/>
+      <c r="AM64" s="155"/>
       <c r="AN64" s="5"/>
       <c r="AO64" s="5"/>
       <c r="AP64" s="5"/>
@@ -6359,12 +6363,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH65" s="144"/>
-      <c r="AI65" s="146"/>
-      <c r="AJ65" s="146"/>
-      <c r="AK65" s="146"/>
-      <c r="AL65" s="146"/>
-      <c r="AM65" s="221"/>
+      <c r="AH65" s="153"/>
+      <c r="AI65" s="154"/>
+      <c r="AJ65" s="154"/>
+      <c r="AK65" s="154"/>
+      <c r="AL65" s="154"/>
+      <c r="AM65" s="155"/>
       <c r="AN65" s="5"/>
       <c r="AO65" s="5"/>
       <c r="AP65" s="5"/>
@@ -6415,12 +6419,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH66" s="144"/>
-      <c r="AI66" s="146"/>
-      <c r="AJ66" s="146"/>
-      <c r="AK66" s="146"/>
-      <c r="AL66" s="146"/>
-      <c r="AM66" s="221"/>
+      <c r="AH66" s="153"/>
+      <c r="AI66" s="154"/>
+      <c r="AJ66" s="154"/>
+      <c r="AK66" s="154"/>
+      <c r="AL66" s="154"/>
+      <c r="AM66" s="155"/>
       <c r="AN66" s="5"/>
       <c r="AO66" s="5"/>
       <c r="AP66" s="5"/>
@@ -6471,12 +6475,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH67" s="144"/>
-      <c r="AI67" s="146"/>
-      <c r="AJ67" s="146"/>
-      <c r="AK67" s="146"/>
-      <c r="AL67" s="146"/>
-      <c r="AM67" s="221"/>
+      <c r="AH67" s="153"/>
+      <c r="AI67" s="154"/>
+      <c r="AJ67" s="154"/>
+      <c r="AK67" s="154"/>
+      <c r="AL67" s="154"/>
+      <c r="AM67" s="155"/>
       <c r="AN67" s="5"/>
       <c r="AO67" s="5"/>
       <c r="AP67" s="5"/>
@@ -6527,12 +6531,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH68" s="144"/>
-      <c r="AI68" s="146"/>
-      <c r="AJ68" s="146"/>
-      <c r="AK68" s="146"/>
-      <c r="AL68" s="146"/>
-      <c r="AM68" s="221"/>
+      <c r="AH68" s="153"/>
+      <c r="AI68" s="154"/>
+      <c r="AJ68" s="154"/>
+      <c r="AK68" s="154"/>
+      <c r="AL68" s="154"/>
+      <c r="AM68" s="155"/>
       <c r="AN68" s="5"/>
       <c r="AO68" s="5"/>
       <c r="AP68" s="5"/>
@@ -6583,12 +6587,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH69" s="148"/>
-      <c r="AI69" s="127"/>
-      <c r="AJ69" s="149"/>
-      <c r="AK69" s="127"/>
-      <c r="AL69" s="127"/>
-      <c r="AM69" s="150"/>
+      <c r="AH69" s="159"/>
+      <c r="AI69" s="136"/>
+      <c r="AJ69" s="160"/>
+      <c r="AK69" s="136"/>
+      <c r="AL69" s="136"/>
+      <c r="AM69" s="161"/>
       <c r="AN69" s="5"/>
       <c r="AO69" s="5"/>
       <c r="AP69" s="5"/>
@@ -6639,12 +6643,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH70" s="148"/>
-      <c r="AI70" s="127"/>
-      <c r="AJ70" s="149"/>
-      <c r="AK70" s="127"/>
-      <c r="AL70" s="127"/>
-      <c r="AM70" s="150"/>
+      <c r="AH70" s="159"/>
+      <c r="AI70" s="136"/>
+      <c r="AJ70" s="160"/>
+      <c r="AK70" s="136"/>
+      <c r="AL70" s="136"/>
+      <c r="AM70" s="161"/>
       <c r="AN70" s="5"/>
       <c r="AO70" s="5"/>
       <c r="AP70" s="5"/>
@@ -6695,12 +6699,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH71" s="148"/>
-      <c r="AI71" s="127"/>
-      <c r="AJ71" s="149"/>
-      <c r="AK71" s="127"/>
-      <c r="AL71" s="127"/>
-      <c r="AM71" s="150"/>
+      <c r="AH71" s="159"/>
+      <c r="AI71" s="136"/>
+      <c r="AJ71" s="160"/>
+      <c r="AK71" s="136"/>
+      <c r="AL71" s="136"/>
+      <c r="AM71" s="161"/>
       <c r="AN71" s="5"/>
       <c r="AO71" s="5"/>
       <c r="AP71" s="5"/>
@@ -6751,12 +6755,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH72" s="148"/>
-      <c r="AI72" s="127"/>
-      <c r="AJ72" s="149"/>
-      <c r="AK72" s="127"/>
-      <c r="AL72" s="127"/>
-      <c r="AM72" s="150"/>
+      <c r="AH72" s="159"/>
+      <c r="AI72" s="136"/>
+      <c r="AJ72" s="160"/>
+      <c r="AK72" s="136"/>
+      <c r="AL72" s="136"/>
+      <c r="AM72" s="161"/>
       <c r="AN72" s="5"/>
       <c r="AO72" s="5"/>
       <c r="AP72" s="5"/>
@@ -6807,12 +6811,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH73" s="148"/>
-      <c r="AI73" s="127"/>
-      <c r="AJ73" s="149"/>
-      <c r="AK73" s="127"/>
-      <c r="AL73" s="127"/>
-      <c r="AM73" s="150"/>
+      <c r="AH73" s="159"/>
+      <c r="AI73" s="136"/>
+      <c r="AJ73" s="160"/>
+      <c r="AK73" s="136"/>
+      <c r="AL73" s="136"/>
+      <c r="AM73" s="161"/>
       <c r="AN73" s="5"/>
       <c r="AO73" s="5"/>
       <c r="AP73" s="5"/>
@@ -6863,12 +6867,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH74" s="148"/>
-      <c r="AI74" s="127"/>
-      <c r="AJ74" s="149"/>
-      <c r="AK74" s="127"/>
-      <c r="AL74" s="127"/>
-      <c r="AM74" s="150"/>
+      <c r="AH74" s="159"/>
+      <c r="AI74" s="136"/>
+      <c r="AJ74" s="160"/>
+      <c r="AK74" s="136"/>
+      <c r="AL74" s="136"/>
+      <c r="AM74" s="161"/>
       <c r="AN74" s="5"/>
       <c r="AO74" s="5"/>
       <c r="AP74" s="5"/>
@@ -6919,12 +6923,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH75" s="148"/>
-      <c r="AI75" s="127"/>
-      <c r="AJ75" s="149"/>
-      <c r="AK75" s="127"/>
-      <c r="AL75" s="127"/>
-      <c r="AM75" s="150"/>
+      <c r="AH75" s="159"/>
+      <c r="AI75" s="136"/>
+      <c r="AJ75" s="160"/>
+      <c r="AK75" s="136"/>
+      <c r="AL75" s="136"/>
+      <c r="AM75" s="161"/>
       <c r="AN75" s="5"/>
       <c r="AO75" s="5"/>
       <c r="AP75" s="5"/>
@@ -6975,12 +6979,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH76" s="148"/>
-      <c r="AI76" s="127"/>
-      <c r="AJ76" s="149"/>
-      <c r="AK76" s="127"/>
-      <c r="AL76" s="127"/>
-      <c r="AM76" s="150"/>
+      <c r="AH76" s="159"/>
+      <c r="AI76" s="136"/>
+      <c r="AJ76" s="160"/>
+      <c r="AK76" s="136"/>
+      <c r="AL76" s="136"/>
+      <c r="AM76" s="161"/>
       <c r="AN76" s="5"/>
       <c r="AO76" s="5"/>
       <c r="AP76" s="5"/>
@@ -7031,12 +7035,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH77" s="148"/>
-      <c r="AI77" s="127"/>
-      <c r="AJ77" s="149"/>
-      <c r="AK77" s="127"/>
-      <c r="AL77" s="127"/>
-      <c r="AM77" s="150"/>
+      <c r="AH77" s="159"/>
+      <c r="AI77" s="136"/>
+      <c r="AJ77" s="160"/>
+      <c r="AK77" s="136"/>
+      <c r="AL77" s="136"/>
+      <c r="AM77" s="161"/>
       <c r="AN77" s="5"/>
       <c r="AO77" s="5"/>
       <c r="AP77" s="5"/>
@@ -7087,12 +7091,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH78" s="148"/>
-      <c r="AI78" s="127"/>
-      <c r="AJ78" s="149"/>
-      <c r="AK78" s="127"/>
-      <c r="AL78" s="127"/>
-      <c r="AM78" s="150"/>
+      <c r="AH78" s="159"/>
+      <c r="AI78" s="136"/>
+      <c r="AJ78" s="160"/>
+      <c r="AK78" s="136"/>
+      <c r="AL78" s="136"/>
+      <c r="AM78" s="161"/>
       <c r="AN78" s="5"/>
       <c r="AO78" s="5"/>
       <c r="AP78" s="5"/>
@@ -7143,12 +7147,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH79" s="148"/>
-      <c r="AI79" s="127"/>
-      <c r="AJ79" s="149"/>
-      <c r="AK79" s="127"/>
-      <c r="AL79" s="127"/>
-      <c r="AM79" s="150"/>
+      <c r="AH79" s="159"/>
+      <c r="AI79" s="136"/>
+      <c r="AJ79" s="160"/>
+      <c r="AK79" s="136"/>
+      <c r="AL79" s="136"/>
+      <c r="AM79" s="161"/>
       <c r="AN79" s="5"/>
       <c r="AO79" s="5"/>
       <c r="AP79" s="5"/>
@@ -7199,12 +7203,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH80" s="148"/>
-      <c r="AI80" s="127"/>
-      <c r="AJ80" s="149"/>
-      <c r="AK80" s="127"/>
-      <c r="AL80" s="127"/>
-      <c r="AM80" s="150"/>
+      <c r="AH80" s="159"/>
+      <c r="AI80" s="136"/>
+      <c r="AJ80" s="160"/>
+      <c r="AK80" s="136"/>
+      <c r="AL80" s="136"/>
+      <c r="AM80" s="161"/>
       <c r="AN80" s="5"/>
       <c r="AO80" s="5"/>
       <c r="AP80" s="5"/>
@@ -7255,12 +7259,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH81" s="148"/>
-      <c r="AI81" s="127"/>
-      <c r="AJ81" s="149"/>
-      <c r="AK81" s="127"/>
-      <c r="AL81" s="127"/>
-      <c r="AM81" s="150"/>
+      <c r="AH81" s="159"/>
+      <c r="AI81" s="136"/>
+      <c r="AJ81" s="160"/>
+      <c r="AK81" s="136"/>
+      <c r="AL81" s="136"/>
+      <c r="AM81" s="161"/>
       <c r="AN81" s="5"/>
       <c r="AO81" s="5"/>
       <c r="AP81" s="5"/>
@@ -7311,8 +7315,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH82" s="148"/>
-      <c r="AI82" s="127"/>
+      <c r="AH82" s="159"/>
+      <c r="AI82" s="136"/>
       <c r="AJ82" s="53"/>
       <c r="AK82" s="53"/>
       <c r="AL82" s="53"/>
@@ -7367,8 +7371,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH83" s="148"/>
-      <c r="AI83" s="127"/>
+      <c r="AH83" s="159"/>
+      <c r="AI83" s="136"/>
       <c r="AJ83" s="53"/>
       <c r="AK83" s="53"/>
       <c r="AL83" s="53"/>
@@ -7423,8 +7427,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH84" s="148"/>
-      <c r="AI84" s="127"/>
+      <c r="AH84" s="159"/>
+      <c r="AI84" s="136"/>
       <c r="AJ84" s="53"/>
       <c r="AK84" s="53"/>
       <c r="AL84" s="53"/>
@@ -7479,8 +7483,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH85" s="148"/>
-      <c r="AI85" s="127"/>
+      <c r="AH85" s="159"/>
+      <c r="AI85" s="136"/>
       <c r="AJ85" s="53"/>
       <c r="AK85" s="53"/>
       <c r="AL85" s="53"/>
@@ -7535,8 +7539,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH86" s="148"/>
-      <c r="AI86" s="127"/>
+      <c r="AH86" s="159"/>
+      <c r="AI86" s="136"/>
       <c r="AJ86" s="53"/>
       <c r="AK86" s="53"/>
       <c r="AL86" s="53"/>
@@ -7591,8 +7595,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH87" s="148"/>
-      <c r="AI87" s="127"/>
+      <c r="AH87" s="159"/>
+      <c r="AI87" s="136"/>
       <c r="AJ87" s="53"/>
       <c r="AK87" s="53"/>
       <c r="AL87" s="53"/>
@@ -7647,8 +7651,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH88" s="148"/>
-      <c r="AI88" s="127"/>
+      <c r="AH88" s="159"/>
+      <c r="AI88" s="136"/>
       <c r="AJ88" s="53"/>
       <c r="AK88" s="53"/>
       <c r="AL88" s="53"/>
@@ -7703,8 +7707,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH89" s="148"/>
-      <c r="AI89" s="127"/>
+      <c r="AH89" s="159"/>
+      <c r="AI89" s="136"/>
       <c r="AJ89" s="53"/>
       <c r="AK89" s="53"/>
       <c r="AL89" s="53"/>
@@ -7759,8 +7763,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH90" s="148"/>
-      <c r="AI90" s="127"/>
+      <c r="AH90" s="159"/>
+      <c r="AI90" s="136"/>
       <c r="AJ90" s="53"/>
       <c r="AK90" s="53"/>
       <c r="AL90" s="53"/>
@@ -7815,8 +7819,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH91" s="148"/>
-      <c r="AI91" s="127"/>
+      <c r="AH91" s="159"/>
+      <c r="AI91" s="136"/>
       <c r="AJ91" s="53"/>
       <c r="AK91" s="53"/>
       <c r="AL91" s="53"/>
@@ -7871,8 +7875,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH92" s="148"/>
-      <c r="AI92" s="127"/>
+      <c r="AH92" s="159"/>
+      <c r="AI92" s="136"/>
       <c r="AJ92" s="53"/>
       <c r="AK92" s="53"/>
       <c r="AL92" s="53"/>
@@ -7927,12 +7931,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH93" s="148"/>
-      <c r="AI93" s="127"/>
-      <c r="AJ93" s="149"/>
-      <c r="AK93" s="127"/>
-      <c r="AL93" s="127"/>
-      <c r="AM93" s="150"/>
+      <c r="AH93" s="159"/>
+      <c r="AI93" s="136"/>
+      <c r="AJ93" s="160"/>
+      <c r="AK93" s="136"/>
+      <c r="AL93" s="136"/>
+      <c r="AM93" s="161"/>
       <c r="AN93" s="5"/>
       <c r="AO93" s="5"/>
       <c r="AP93" s="5"/>
@@ -7983,8 +7987,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH94" s="148"/>
-      <c r="AI94" s="127"/>
+      <c r="AH94" s="159"/>
+      <c r="AI94" s="136"/>
       <c r="AJ94" s="53"/>
       <c r="AK94" s="53"/>
       <c r="AL94" s="53"/>
@@ -8039,8 +8043,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH95" s="148"/>
-      <c r="AI95" s="127"/>
+      <c r="AH95" s="159"/>
+      <c r="AI95" s="136"/>
       <c r="AJ95" s="53"/>
       <c r="AK95" s="53"/>
       <c r="AL95" s="53"/>
@@ -8095,8 +8099,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH96" s="148"/>
-      <c r="AI96" s="127"/>
+      <c r="AH96" s="159"/>
+      <c r="AI96" s="136"/>
       <c r="AJ96" s="53"/>
       <c r="AK96" s="53"/>
       <c r="AL96" s="53"/>
@@ -8151,8 +8155,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH97" s="148"/>
-      <c r="AI97" s="127"/>
+      <c r="AH97" s="159"/>
+      <c r="AI97" s="136"/>
       <c r="AJ97" s="53"/>
       <c r="AK97" s="53"/>
       <c r="AL97" s="53"/>
@@ -8207,8 +8211,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH98" s="148"/>
-      <c r="AI98" s="127"/>
+      <c r="AH98" s="159"/>
+      <c r="AI98" s="136"/>
       <c r="AJ98" s="53"/>
       <c r="AK98" s="53"/>
       <c r="AL98" s="53"/>
@@ -8263,8 +8267,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH99" s="148"/>
-      <c r="AI99" s="127"/>
+      <c r="AH99" s="159"/>
+      <c r="AI99" s="136"/>
       <c r="AJ99" s="53"/>
       <c r="AK99" s="53"/>
       <c r="AL99" s="53"/>
@@ -8319,8 +8323,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH100" s="148"/>
-      <c r="AI100" s="127"/>
+      <c r="AH100" s="159"/>
+      <c r="AI100" s="136"/>
       <c r="AJ100" s="53"/>
       <c r="AK100" s="53"/>
       <c r="AL100" s="53"/>
@@ -8375,8 +8379,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH101" s="148"/>
-      <c r="AI101" s="127"/>
+      <c r="AH101" s="159"/>
+      <c r="AI101" s="136"/>
       <c r="AJ101" s="53"/>
       <c r="AK101" s="53"/>
       <c r="AL101" s="53"/>
@@ -8431,8 +8435,8 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH102" s="148"/>
-      <c r="AI102" s="127"/>
+      <c r="AH102" s="159"/>
+      <c r="AI102" s="136"/>
       <c r="AJ102" s="53"/>
       <c r="AK102" s="53"/>
       <c r="AL102" s="53"/>
@@ -8487,12 +8491,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH103" s="148"/>
-      <c r="AI103" s="127"/>
-      <c r="AJ103" s="149"/>
-      <c r="AK103" s="127"/>
-      <c r="AL103" s="127"/>
-      <c r="AM103" s="150"/>
+      <c r="AH103" s="159"/>
+      <c r="AI103" s="136"/>
+      <c r="AJ103" s="160"/>
+      <c r="AK103" s="136"/>
+      <c r="AL103" s="136"/>
+      <c r="AM103" s="161"/>
       <c r="AN103" s="5"/>
       <c r="AO103" s="5"/>
       <c r="AP103" s="5"/>
@@ -8543,12 +8547,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH104" s="148"/>
-      <c r="AI104" s="127"/>
-      <c r="AJ104" s="149"/>
-      <c r="AK104" s="127"/>
-      <c r="AL104" s="127"/>
-      <c r="AM104" s="150"/>
+      <c r="AH104" s="159"/>
+      <c r="AI104" s="136"/>
+      <c r="AJ104" s="160"/>
+      <c r="AK104" s="136"/>
+      <c r="AL104" s="136"/>
+      <c r="AM104" s="161"/>
       <c r="AN104" s="5"/>
       <c r="AO104" s="5"/>
       <c r="AP104" s="5"/>
@@ -8599,12 +8603,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH105" s="148"/>
-      <c r="AI105" s="127"/>
-      <c r="AJ105" s="149"/>
-      <c r="AK105" s="127"/>
-      <c r="AL105" s="127"/>
-      <c r="AM105" s="150"/>
+      <c r="AH105" s="159"/>
+      <c r="AI105" s="136"/>
+      <c r="AJ105" s="160"/>
+      <c r="AK105" s="136"/>
+      <c r="AL105" s="136"/>
+      <c r="AM105" s="161"/>
       <c r="AN105" s="5"/>
       <c r="AO105" s="5"/>
       <c r="AP105" s="5"/>
@@ -8655,12 +8659,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH106" s="148"/>
-      <c r="AI106" s="127"/>
-      <c r="AJ106" s="149"/>
-      <c r="AK106" s="127"/>
-      <c r="AL106" s="127"/>
-      <c r="AM106" s="150"/>
+      <c r="AH106" s="159"/>
+      <c r="AI106" s="136"/>
+      <c r="AJ106" s="160"/>
+      <c r="AK106" s="136"/>
+      <c r="AL106" s="136"/>
+      <c r="AM106" s="161"/>
       <c r="AN106" s="5"/>
       <c r="AO106" s="5"/>
       <c r="AP106" s="5"/>
@@ -8711,12 +8715,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH107" s="148"/>
-      <c r="AI107" s="127"/>
-      <c r="AJ107" s="149"/>
-      <c r="AK107" s="127"/>
-      <c r="AL107" s="127"/>
-      <c r="AM107" s="150"/>
+      <c r="AH107" s="159"/>
+      <c r="AI107" s="136"/>
+      <c r="AJ107" s="160"/>
+      <c r="AK107" s="136"/>
+      <c r="AL107" s="136"/>
+      <c r="AM107" s="161"/>
       <c r="AN107" s="5"/>
       <c r="AO107" s="5"/>
       <c r="AP107" s="5"/>
@@ -8767,12 +8771,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH108" s="148"/>
-      <c r="AI108" s="127"/>
-      <c r="AJ108" s="149"/>
-      <c r="AK108" s="127"/>
-      <c r="AL108" s="127"/>
-      <c r="AM108" s="150"/>
+      <c r="AH108" s="159"/>
+      <c r="AI108" s="136"/>
+      <c r="AJ108" s="160"/>
+      <c r="AK108" s="136"/>
+      <c r="AL108" s="136"/>
+      <c r="AM108" s="161"/>
       <c r="AN108" s="5"/>
       <c r="AO108" s="5"/>
       <c r="AP108" s="5"/>
@@ -8823,12 +8827,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH109" s="148"/>
-      <c r="AI109" s="127"/>
-      <c r="AJ109" s="149"/>
-      <c r="AK109" s="127"/>
-      <c r="AL109" s="127"/>
-      <c r="AM109" s="150"/>
+      <c r="AH109" s="159"/>
+      <c r="AI109" s="136"/>
+      <c r="AJ109" s="160"/>
+      <c r="AK109" s="136"/>
+      <c r="AL109" s="136"/>
+      <c r="AM109" s="161"/>
       <c r="AN109" s="5"/>
       <c r="AO109" s="5"/>
       <c r="AP109" s="5"/>
@@ -8879,12 +8883,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH110" s="148"/>
-      <c r="AI110" s="127"/>
-      <c r="AJ110" s="149"/>
-      <c r="AK110" s="127"/>
-      <c r="AL110" s="127"/>
-      <c r="AM110" s="150"/>
+      <c r="AH110" s="159"/>
+      <c r="AI110" s="136"/>
+      <c r="AJ110" s="160"/>
+      <c r="AK110" s="136"/>
+      <c r="AL110" s="136"/>
+      <c r="AM110" s="161"/>
       <c r="AN110" s="5"/>
       <c r="AO110" s="5"/>
       <c r="AP110" s="5"/>
@@ -8935,12 +8939,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH111" s="148"/>
-      <c r="AI111" s="127"/>
-      <c r="AJ111" s="149"/>
-      <c r="AK111" s="127"/>
-      <c r="AL111" s="127"/>
-      <c r="AM111" s="150"/>
+      <c r="AH111" s="159"/>
+      <c r="AI111" s="136"/>
+      <c r="AJ111" s="160"/>
+      <c r="AK111" s="136"/>
+      <c r="AL111" s="136"/>
+      <c r="AM111" s="161"/>
       <c r="AN111" s="5"/>
       <c r="AO111" s="5"/>
       <c r="AP111" s="5"/>
@@ -8991,12 +8995,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH112" s="148"/>
-      <c r="AI112" s="127"/>
-      <c r="AJ112" s="149"/>
-      <c r="AK112" s="127"/>
-      <c r="AL112" s="127"/>
-      <c r="AM112" s="150"/>
+      <c r="AH112" s="159"/>
+      <c r="AI112" s="136"/>
+      <c r="AJ112" s="160"/>
+      <c r="AK112" s="136"/>
+      <c r="AL112" s="136"/>
+      <c r="AM112" s="161"/>
       <c r="AN112" s="5"/>
       <c r="AO112" s="5"/>
       <c r="AP112" s="5"/>
@@ -9047,12 +9051,12 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="AH113" s="148"/>
-      <c r="AI113" s="127"/>
-      <c r="AJ113" s="163"/>
-      <c r="AK113" s="164"/>
-      <c r="AL113" s="164"/>
-      <c r="AM113" s="165"/>
+      <c r="AH113" s="159"/>
+      <c r="AI113" s="136"/>
+      <c r="AJ113" s="162"/>
+      <c r="AK113" s="163"/>
+      <c r="AL113" s="163"/>
+      <c r="AM113" s="164"/>
       <c r="AN113" s="5"/>
       <c r="AO113" s="5"/>
       <c r="AP113" s="5"/>
@@ -9062,10 +9066,10 @@
       <c r="AT113" s="5"/>
     </row>
     <row r="114" spans="1:46" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="166" t="s">
+      <c r="A114" s="165" t="s">
         <v>32</v>
       </c>
-      <c r="B114" s="155"/>
+      <c r="B114" s="145"/>
       <c r="C114" s="63"/>
       <c r="D114" s="63"/>
       <c r="E114" s="63"/>
@@ -9178,12 +9182,12 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AH114" s="167"/>
-      <c r="AI114" s="155"/>
-      <c r="AJ114" s="155"/>
-      <c r="AK114" s="155"/>
-      <c r="AL114" s="155"/>
-      <c r="AM114" s="156"/>
+      <c r="AH114" s="166"/>
+      <c r="AI114" s="145"/>
+      <c r="AJ114" s="145"/>
+      <c r="AK114" s="145"/>
+      <c r="AL114" s="145"/>
+      <c r="AM114" s="146"/>
       <c r="AN114" s="5"/>
       <c r="AO114" s="5"/>
       <c r="AP114" s="5"/>
@@ -9193,10 +9197,10 @@
       <c r="AT114" s="5"/>
     </row>
     <row r="115" spans="1:46" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A115" s="177" t="s">
+      <c r="A115" s="176" t="s">
         <v>33</v>
       </c>
-      <c r="B115" s="135"/>
+      <c r="B115" s="126"/>
       <c r="C115" s="81"/>
       <c r="D115" s="81"/>
       <c r="E115" s="81"/>
@@ -9309,12 +9313,12 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AH115" s="178"/>
-      <c r="AI115" s="158"/>
-      <c r="AJ115" s="158"/>
-      <c r="AK115" s="158"/>
-      <c r="AL115" s="158"/>
-      <c r="AM115" s="139"/>
+      <c r="AH115" s="177"/>
+      <c r="AI115" s="148"/>
+      <c r="AJ115" s="148"/>
+      <c r="AK115" s="148"/>
+      <c r="AL115" s="148"/>
+      <c r="AM115" s="130"/>
       <c r="AN115" s="5"/>
       <c r="AO115" s="5"/>
       <c r="AP115" s="5"/>
@@ -9324,17 +9328,17 @@
       <c r="AT115" s="5"/>
     </row>
     <row r="116" spans="1:46" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A116" s="179"/>
-      <c r="B116" s="124"/>
+      <c r="A116" s="178"/>
+      <c r="B116" s="134"/>
       <c r="C116" s="87"/>
       <c r="D116" s="87"/>
       <c r="E116" s="87"/>
       <c r="F116" s="87"/>
-      <c r="G116" s="180"/>
-      <c r="H116" s="124"/>
-      <c r="I116" s="124"/>
-      <c r="J116" s="124"/>
-      <c r="K116" s="124"/>
+      <c r="G116" s="179"/>
+      <c r="H116" s="134"/>
+      <c r="I116" s="134"/>
+      <c r="J116" s="134"/>
+      <c r="K116" s="134"/>
       <c r="L116" s="5"/>
       <c r="M116" s="5"/>
       <c r="N116" s="5"/>
@@ -9406,27 +9410,27 @@
       <c r="AB117" s="95"/>
       <c r="AC117" s="96"/>
       <c r="AD117" s="5"/>
-      <c r="AE117" s="181" t="s">
+      <c r="AE117" s="180" t="s">
         <v>36</v>
       </c>
-      <c r="AF117" s="152"/>
-      <c r="AG117" s="182" t="str">
+      <c r="AF117" s="142"/>
+      <c r="AG117" s="181" t="str">
         <f>AA6</f>
         <v>(Month)</v>
       </c>
-      <c r="AH117" s="183" t="s">
+      <c r="AH117" s="182" t="s">
         <v>37</v>
       </c>
-      <c r="AI117" s="152"/>
-      <c r="AJ117" s="184">
+      <c r="AI117" s="142"/>
+      <c r="AJ117" s="183">
         <f>AQ9</f>
         <v>16</v>
       </c>
-      <c r="AK117" s="185" t="s">
+      <c r="AK117" s="184" t="s">
         <v>38</v>
       </c>
-      <c r="AL117" s="145"/>
-      <c r="AM117" s="147"/>
+      <c r="AL117" s="185"/>
+      <c r="AM117" s="186"/>
       <c r="AN117" s="5"/>
       <c r="AO117" s="5"/>
       <c r="AP117" s="5"/>
@@ -9436,46 +9440,46 @@
       <c r="AT117" s="5"/>
     </row>
     <row r="118" spans="1:46" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A118" s="169" t="s">
+      <c r="A118" s="168" t="s">
         <v>39</v>
       </c>
-      <c r="B118" s="124"/>
-      <c r="C118" s="124"/>
-      <c r="D118" s="124"/>
-      <c r="E118" s="124"/>
-      <c r="F118" s="124"/>
-      <c r="G118" s="124"/>
-      <c r="H118" s="124"/>
-      <c r="I118" s="124"/>
-      <c r="J118" s="124"/>
-      <c r="K118" s="124"/>
-      <c r="L118" s="124"/>
-      <c r="M118" s="124"/>
-      <c r="N118" s="124"/>
-      <c r="O118" s="124"/>
-      <c r="P118" s="124"/>
-      <c r="Q118" s="124"/>
+      <c r="B118" s="134"/>
+      <c r="C118" s="134"/>
+      <c r="D118" s="134"/>
+      <c r="E118" s="134"/>
+      <c r="F118" s="134"/>
+      <c r="G118" s="134"/>
+      <c r="H118" s="134"/>
+      <c r="I118" s="134"/>
+      <c r="J118" s="134"/>
+      <c r="K118" s="134"/>
+      <c r="L118" s="134"/>
+      <c r="M118" s="134"/>
+      <c r="N118" s="134"/>
+      <c r="O118" s="134"/>
+      <c r="P118" s="134"/>
+      <c r="Q118" s="134"/>
       <c r="R118" s="90"/>
       <c r="S118" s="91"/>
-      <c r="T118" s="168" t="s">
+      <c r="T118" s="167" t="s">
         <v>40</v>
       </c>
-      <c r="U118" s="152"/>
-      <c r="V118" s="152"/>
-      <c r="W118" s="152"/>
-      <c r="X118" s="152"/>
-      <c r="Y118" s="152"/>
-      <c r="Z118" s="152"/>
-      <c r="AA118" s="152"/>
-      <c r="AB118" s="152"/>
+      <c r="U118" s="142"/>
+      <c r="V118" s="142"/>
+      <c r="W118" s="142"/>
+      <c r="X118" s="142"/>
+      <c r="Y118" s="142"/>
+      <c r="Z118" s="142"/>
+      <c r="AA118" s="142"/>
+      <c r="AB118" s="142"/>
       <c r="AC118" s="97"/>
       <c r="AD118" s="5"/>
-      <c r="AE118" s="162"/>
-      <c r="AF118" s="158"/>
-      <c r="AG118" s="139"/>
-      <c r="AH118" s="162"/>
-      <c r="AI118" s="158"/>
-      <c r="AJ118" s="139"/>
+      <c r="AE118" s="152"/>
+      <c r="AF118" s="148"/>
+      <c r="AG118" s="130"/>
+      <c r="AH118" s="152"/>
+      <c r="AI118" s="148"/>
+      <c r="AJ118" s="130"/>
       <c r="AK118" s="98" t="s">
         <v>14</v>
       </c>
@@ -9494,53 +9498,53 @@
       <c r="AT118" s="5"/>
     </row>
     <row r="119" spans="1:46" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="169" t="s">
+      <c r="A119" s="168" t="s">
         <v>42</v>
       </c>
-      <c r="B119" s="124"/>
-      <c r="C119" s="124"/>
-      <c r="D119" s="124"/>
-      <c r="E119" s="124"/>
-      <c r="F119" s="124"/>
-      <c r="G119" s="124"/>
-      <c r="H119" s="124"/>
-      <c r="I119" s="124"/>
-      <c r="J119" s="124"/>
-      <c r="K119" s="124"/>
-      <c r="L119" s="124"/>
-      <c r="M119" s="124"/>
-      <c r="N119" s="124"/>
-      <c r="O119" s="124"/>
-      <c r="P119" s="124"/>
-      <c r="Q119" s="124"/>
+      <c r="B119" s="134"/>
+      <c r="C119" s="134"/>
+      <c r="D119" s="134"/>
+      <c r="E119" s="134"/>
+      <c r="F119" s="134"/>
+      <c r="G119" s="134"/>
+      <c r="H119" s="134"/>
+      <c r="I119" s="134"/>
+      <c r="J119" s="134"/>
+      <c r="K119" s="134"/>
+      <c r="L119" s="134"/>
+      <c r="M119" s="134"/>
+      <c r="N119" s="134"/>
+      <c r="O119" s="134"/>
+      <c r="P119" s="134"/>
+      <c r="Q119" s="134"/>
       <c r="R119" s="90"/>
       <c r="S119" s="91"/>
-      <c r="T119" s="153"/>
-      <c r="U119" s="124"/>
-      <c r="V119" s="124"/>
-      <c r="W119" s="124"/>
-      <c r="X119" s="124"/>
-      <c r="Y119" s="124"/>
-      <c r="Z119" s="124"/>
-      <c r="AA119" s="124"/>
-      <c r="AB119" s="124"/>
+      <c r="T119" s="143"/>
+      <c r="U119" s="134"/>
+      <c r="V119" s="134"/>
+      <c r="W119" s="134"/>
+      <c r="X119" s="134"/>
+      <c r="Y119" s="134"/>
+      <c r="Z119" s="134"/>
+      <c r="AA119" s="134"/>
+      <c r="AB119" s="134"/>
       <c r="AC119" s="97"/>
       <c r="AD119" s="5"/>
-      <c r="AE119" s="170" t="s">
+      <c r="AE119" s="169" t="s">
         <v>43</v>
       </c>
-      <c r="AF119" s="152"/>
-      <c r="AG119" s="152"/>
-      <c r="AH119" s="152"/>
-      <c r="AI119" s="152"/>
-      <c r="AJ119" s="171"/>
-      <c r="AK119" s="174">
+      <c r="AF119" s="142"/>
+      <c r="AG119" s="142"/>
+      <c r="AH119" s="142"/>
+      <c r="AI119" s="142"/>
+      <c r="AJ119" s="170"/>
+      <c r="AK119" s="173">
         <v>11</v>
       </c>
-      <c r="AL119" s="174">
+      <c r="AL119" s="173">
         <v>5</v>
       </c>
-      <c r="AM119" s="175">
+      <c r="AM119" s="174">
         <f>AK119+AL119</f>
         <v>16</v>
       </c>
@@ -9553,47 +9557,47 @@
       <c r="AT119" s="5"/>
     </row>
     <row r="120" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="169" t="s">
+      <c r="A120" s="168" t="s">
         <v>44</v>
       </c>
-      <c r="B120" s="124"/>
-      <c r="C120" s="124"/>
-      <c r="D120" s="124"/>
-      <c r="E120" s="124"/>
-      <c r="F120" s="124"/>
-      <c r="G120" s="124"/>
-      <c r="H120" s="124"/>
-      <c r="I120" s="124"/>
-      <c r="J120" s="124"/>
-      <c r="K120" s="124"/>
-      <c r="L120" s="124"/>
-      <c r="M120" s="124"/>
-      <c r="N120" s="124"/>
-      <c r="O120" s="124"/>
-      <c r="P120" s="124"/>
-      <c r="Q120" s="124"/>
+      <c r="B120" s="134"/>
+      <c r="C120" s="134"/>
+      <c r="D120" s="134"/>
+      <c r="E120" s="134"/>
+      <c r="F120" s="134"/>
+      <c r="G120" s="134"/>
+      <c r="H120" s="134"/>
+      <c r="I120" s="134"/>
+      <c r="J120" s="134"/>
+      <c r="K120" s="134"/>
+      <c r="L120" s="134"/>
+      <c r="M120" s="134"/>
+      <c r="N120" s="134"/>
+      <c r="O120" s="134"/>
+      <c r="P120" s="134"/>
+      <c r="Q120" s="134"/>
       <c r="R120" s="90"/>
       <c r="S120" s="91"/>
-      <c r="T120" s="153"/>
-      <c r="U120" s="124"/>
-      <c r="V120" s="124"/>
-      <c r="W120" s="124"/>
-      <c r="X120" s="124"/>
-      <c r="Y120" s="124"/>
-      <c r="Z120" s="124"/>
-      <c r="AA120" s="124"/>
-      <c r="AB120" s="124"/>
+      <c r="T120" s="143"/>
+      <c r="U120" s="134"/>
+      <c r="V120" s="134"/>
+      <c r="W120" s="134"/>
+      <c r="X120" s="134"/>
+      <c r="Y120" s="134"/>
+      <c r="Z120" s="134"/>
+      <c r="AA120" s="134"/>
+      <c r="AB120" s="134"/>
       <c r="AC120" s="97"/>
       <c r="AD120" s="5"/>
-      <c r="AE120" s="172"/>
-      <c r="AF120" s="173"/>
-      <c r="AG120" s="173"/>
-      <c r="AH120" s="173"/>
-      <c r="AI120" s="173"/>
-      <c r="AJ120" s="135"/>
-      <c r="AK120" s="137"/>
-      <c r="AL120" s="137"/>
-      <c r="AM120" s="176"/>
+      <c r="AE120" s="171"/>
+      <c r="AF120" s="172"/>
+      <c r="AG120" s="172"/>
+      <c r="AH120" s="172"/>
+      <c r="AI120" s="172"/>
+      <c r="AJ120" s="126"/>
+      <c r="AK120" s="128"/>
+      <c r="AL120" s="128"/>
+      <c r="AM120" s="175"/>
       <c r="AN120" s="5"/>
       <c r="AO120" s="5"/>
       <c r="AP120" s="5"/>
@@ -9603,32 +9607,32 @@
       <c r="AT120" s="5"/>
     </row>
     <row r="121" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="190" t="s">
+      <c r="A121" s="191" t="s">
         <v>45</v>
       </c>
-      <c r="B121" s="195" t="s">
+      <c r="B121" s="196" t="s">
         <v>46</v>
       </c>
       <c r="C121" s="102"/>
       <c r="D121" s="102"/>
       <c r="E121" s="102"/>
       <c r="F121" s="102"/>
-      <c r="G121" s="196" t="s">
+      <c r="G121" s="197" t="s">
         <v>47</v>
       </c>
-      <c r="H121" s="173"/>
-      <c r="I121" s="173"/>
-      <c r="J121" s="173"/>
-      <c r="K121" s="173"/>
-      <c r="L121" s="173"/>
-      <c r="M121" s="173"/>
-      <c r="N121" s="173"/>
-      <c r="O121" s="173"/>
-      <c r="P121" s="173"/>
-      <c r="Q121" s="197" t="s">
+      <c r="H121" s="172"/>
+      <c r="I121" s="172"/>
+      <c r="J121" s="172"/>
+      <c r="K121" s="172"/>
+      <c r="L121" s="172"/>
+      <c r="M121" s="172"/>
+      <c r="N121" s="172"/>
+      <c r="O121" s="172"/>
+      <c r="P121" s="172"/>
+      <c r="Q121" s="198" t="s">
         <v>48</v>
       </c>
-      <c r="R121" s="124"/>
+      <c r="R121" s="134"/>
       <c r="S121" s="91"/>
       <c r="T121" s="104" t="s">
         <v>49</v>
@@ -9643,21 +9647,21 @@
       <c r="AB121" s="105"/>
       <c r="AC121" s="97"/>
       <c r="AD121" s="5"/>
-      <c r="AE121" s="193" t="s">
+      <c r="AE121" s="194" t="s">
         <v>50</v>
       </c>
-      <c r="AF121" s="189"/>
-      <c r="AG121" s="189"/>
-      <c r="AH121" s="189"/>
-      <c r="AI121" s="189"/>
-      <c r="AJ121" s="133"/>
-      <c r="AK121" s="186">
+      <c r="AF121" s="190"/>
+      <c r="AG121" s="190"/>
+      <c r="AH121" s="190"/>
+      <c r="AI121" s="190"/>
+      <c r="AJ121" s="124"/>
+      <c r="AK121" s="187">
         <v>0</v>
       </c>
-      <c r="AL121" s="186">
+      <c r="AL121" s="187">
         <v>0</v>
       </c>
-      <c r="AM121" s="187">
+      <c r="AM121" s="188">
         <f>AK121+AL121</f>
         <v>0</v>
       </c>
@@ -9670,26 +9674,26 @@
       <c r="AT121" s="5"/>
     </row>
     <row r="122" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="124"/>
-      <c r="B122" s="124"/>
+      <c r="A122" s="134"/>
+      <c r="B122" s="134"/>
       <c r="C122" s="102"/>
       <c r="D122" s="102"/>
       <c r="E122" s="102"/>
       <c r="F122" s="102"/>
-      <c r="G122" s="188" t="s">
+      <c r="G122" s="189" t="s">
         <v>51</v>
       </c>
-      <c r="H122" s="189"/>
-      <c r="I122" s="189"/>
-      <c r="J122" s="189"/>
-      <c r="K122" s="189"/>
-      <c r="L122" s="189"/>
-      <c r="M122" s="189"/>
-      <c r="N122" s="189"/>
-      <c r="O122" s="189"/>
-      <c r="P122" s="189"/>
-      <c r="Q122" s="124"/>
-      <c r="R122" s="124"/>
+      <c r="H122" s="190"/>
+      <c r="I122" s="190"/>
+      <c r="J122" s="190"/>
+      <c r="K122" s="190"/>
+      <c r="L122" s="190"/>
+      <c r="M122" s="190"/>
+      <c r="N122" s="190"/>
+      <c r="O122" s="190"/>
+      <c r="P122" s="190"/>
+      <c r="Q122" s="134"/>
+      <c r="R122" s="134"/>
       <c r="S122" s="91"/>
       <c r="T122" s="104" t="s">
         <v>52</v>
@@ -9704,15 +9708,15 @@
       <c r="AB122" s="105"/>
       <c r="AC122" s="97"/>
       <c r="AD122" s="5"/>
-      <c r="AE122" s="172"/>
-      <c r="AF122" s="173"/>
-      <c r="AG122" s="173"/>
-      <c r="AH122" s="173"/>
-      <c r="AI122" s="173"/>
-      <c r="AJ122" s="135"/>
-      <c r="AK122" s="137"/>
-      <c r="AL122" s="137"/>
-      <c r="AM122" s="176"/>
+      <c r="AE122" s="171"/>
+      <c r="AF122" s="172"/>
+      <c r="AG122" s="172"/>
+      <c r="AH122" s="172"/>
+      <c r="AI122" s="172"/>
+      <c r="AJ122" s="126"/>
+      <c r="AK122" s="128"/>
+      <c r="AL122" s="128"/>
+      <c r="AM122" s="175"/>
       <c r="AN122" s="5"/>
       <c r="AO122" s="5"/>
       <c r="AP122" s="5"/>
@@ -9722,28 +9726,28 @@
       <c r="AT122" s="5"/>
     </row>
     <row r="123" spans="1:46" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="190" t="s">
+      <c r="A123" s="191" t="s">
         <v>53</v>
       </c>
-      <c r="B123" s="191" t="s">
+      <c r="B123" s="192" t="s">
         <v>54</v>
       </c>
       <c r="C123" s="106"/>
       <c r="D123" s="106"/>
       <c r="E123" s="106"/>
       <c r="F123" s="106"/>
-      <c r="G123" s="192" t="s">
+      <c r="G123" s="193" t="s">
         <v>55</v>
       </c>
-      <c r="H123" s="173"/>
-      <c r="I123" s="173"/>
-      <c r="J123" s="173"/>
-      <c r="K123" s="173"/>
-      <c r="L123" s="173"/>
-      <c r="M123" s="173"/>
-      <c r="N123" s="173"/>
-      <c r="O123" s="173"/>
-      <c r="P123" s="173"/>
+      <c r="H123" s="172"/>
+      <c r="I123" s="172"/>
+      <c r="J123" s="172"/>
+      <c r="K123" s="172"/>
+      <c r="L123" s="172"/>
+      <c r="M123" s="172"/>
+      <c r="N123" s="172"/>
+      <c r="O123" s="172"/>
+      <c r="P123" s="172"/>
       <c r="Q123" s="107"/>
       <c r="R123" s="90"/>
       <c r="S123" s="91"/>
@@ -9760,23 +9764,23 @@
       <c r="AB123" s="105"/>
       <c r="AC123" s="97"/>
       <c r="AD123" s="5"/>
-      <c r="AE123" s="193" t="s">
+      <c r="AE123" s="194" t="s">
         <v>57</v>
       </c>
-      <c r="AF123" s="189"/>
-      <c r="AG123" s="189"/>
-      <c r="AH123" s="189"/>
-      <c r="AI123" s="189"/>
-      <c r="AJ123" s="133"/>
-      <c r="AK123" s="194">
+      <c r="AF123" s="190"/>
+      <c r="AG123" s="190"/>
+      <c r="AH123" s="190"/>
+      <c r="AI123" s="190"/>
+      <c r="AJ123" s="124"/>
+      <c r="AK123" s="195">
         <f>COUNTA($B$13:$B$62)</f>
         <v>0</v>
       </c>
-      <c r="AL123" s="194">
+      <c r="AL123" s="195">
         <f>COUNTA($B$64:$B$113)</f>
         <v>0</v>
       </c>
-      <c r="AM123" s="175">
+      <c r="AM123" s="174">
         <f>AK123+AL123</f>
         <v>0</v>
       </c>
@@ -9789,24 +9793,24 @@
       <c r="AT123" s="5"/>
     </row>
     <row r="124" spans="1:46" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="124"/>
-      <c r="B124" s="124"/>
+      <c r="A124" s="134"/>
+      <c r="B124" s="134"/>
       <c r="C124" s="106"/>
       <c r="D124" s="106"/>
       <c r="E124" s="106"/>
       <c r="F124" s="106"/>
-      <c r="G124" s="188" t="s">
+      <c r="G124" s="189" t="s">
         <v>58</v>
       </c>
-      <c r="H124" s="189"/>
-      <c r="I124" s="189"/>
-      <c r="J124" s="189"/>
-      <c r="K124" s="189"/>
-      <c r="L124" s="189"/>
-      <c r="M124" s="189"/>
-      <c r="N124" s="189"/>
-      <c r="O124" s="189"/>
-      <c r="P124" s="189"/>
+      <c r="H124" s="190"/>
+      <c r="I124" s="190"/>
+      <c r="J124" s="190"/>
+      <c r="K124" s="190"/>
+      <c r="L124" s="190"/>
+      <c r="M124" s="190"/>
+      <c r="N124" s="190"/>
+      <c r="O124" s="190"/>
+      <c r="P124" s="190"/>
       <c r="Q124" s="90"/>
       <c r="R124" s="90"/>
       <c r="S124" s="91"/>
@@ -9823,15 +9827,15 @@
       <c r="AB124" s="105"/>
       <c r="AC124" s="97"/>
       <c r="AD124" s="5"/>
-      <c r="AE124" s="172"/>
-      <c r="AF124" s="173"/>
-      <c r="AG124" s="173"/>
-      <c r="AH124" s="173"/>
-      <c r="AI124" s="173"/>
-      <c r="AJ124" s="135"/>
-      <c r="AK124" s="137"/>
-      <c r="AL124" s="137"/>
-      <c r="AM124" s="176"/>
+      <c r="AE124" s="171"/>
+      <c r="AF124" s="172"/>
+      <c r="AG124" s="172"/>
+      <c r="AH124" s="172"/>
+      <c r="AI124" s="172"/>
+      <c r="AJ124" s="126"/>
+      <c r="AK124" s="128"/>
+      <c r="AL124" s="128"/>
+      <c r="AM124" s="175"/>
       <c r="AN124" s="5"/>
       <c r="AO124" s="5"/>
       <c r="AP124" s="5"/>
@@ -9841,32 +9845,32 @@
       <c r="AT124" s="5"/>
     </row>
     <row r="125" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="201" t="s">
+      <c r="A125" s="202" t="s">
         <v>60</v>
       </c>
-      <c r="B125" s="195" t="s">
+      <c r="B125" s="196" t="s">
         <v>61</v>
       </c>
       <c r="C125" s="102"/>
       <c r="D125" s="102"/>
       <c r="E125" s="102"/>
       <c r="F125" s="102"/>
-      <c r="G125" s="196" t="s">
+      <c r="G125" s="197" t="s">
         <v>62</v>
       </c>
-      <c r="H125" s="173"/>
-      <c r="I125" s="173"/>
-      <c r="J125" s="173"/>
-      <c r="K125" s="173"/>
-      <c r="L125" s="173"/>
-      <c r="M125" s="173"/>
-      <c r="N125" s="173"/>
-      <c r="O125" s="173"/>
-      <c r="P125" s="173"/>
-      <c r="Q125" s="197" t="s">
+      <c r="H125" s="172"/>
+      <c r="I125" s="172"/>
+      <c r="J125" s="172"/>
+      <c r="K125" s="172"/>
+      <c r="L125" s="172"/>
+      <c r="M125" s="172"/>
+      <c r="N125" s="172"/>
+      <c r="O125" s="172"/>
+      <c r="P125" s="172"/>
+      <c r="Q125" s="198" t="s">
         <v>48</v>
       </c>
-      <c r="R125" s="124"/>
+      <c r="R125" s="134"/>
       <c r="S125" s="91"/>
       <c r="T125" s="108" t="s">
         <v>63</v>
@@ -9881,23 +9885,23 @@
       <c r="AB125" s="105"/>
       <c r="AC125" s="97"/>
       <c r="AD125" s="5"/>
-      <c r="AE125" s="202" t="s">
+      <c r="AE125" s="203" t="s">
         <v>64</v>
       </c>
-      <c r="AF125" s="189"/>
-      <c r="AG125" s="189"/>
-      <c r="AH125" s="189"/>
-      <c r="AI125" s="189"/>
-      <c r="AJ125" s="133"/>
-      <c r="AK125" s="198">
+      <c r="AF125" s="190"/>
+      <c r="AG125" s="190"/>
+      <c r="AH125" s="190"/>
+      <c r="AI125" s="190"/>
+      <c r="AJ125" s="124"/>
+      <c r="AK125" s="199">
         <f t="shared" ref="AK125:AM125" si="10">AK123/AK119</f>
         <v>0</v>
       </c>
-      <c r="AL125" s="198">
+      <c r="AL125" s="199">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="AM125" s="199">
+      <c r="AM125" s="200">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
@@ -9910,26 +9914,26 @@
       <c r="AT125" s="5"/>
     </row>
     <row r="126" spans="1:46" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="124"/>
-      <c r="B126" s="124"/>
+      <c r="A126" s="134"/>
+      <c r="B126" s="134"/>
       <c r="C126" s="102"/>
       <c r="D126" s="102"/>
       <c r="E126" s="102"/>
       <c r="F126" s="102"/>
-      <c r="G126" s="197" t="s">
+      <c r="G126" s="198" t="s">
         <v>65</v>
       </c>
-      <c r="H126" s="124"/>
-      <c r="I126" s="124"/>
-      <c r="J126" s="124"/>
-      <c r="K126" s="124"/>
-      <c r="L126" s="124"/>
-      <c r="M126" s="124"/>
-      <c r="N126" s="124"/>
-      <c r="O126" s="124"/>
-      <c r="P126" s="124"/>
-      <c r="Q126" s="124"/>
-      <c r="R126" s="124"/>
+      <c r="H126" s="134"/>
+      <c r="I126" s="134"/>
+      <c r="J126" s="134"/>
+      <c r="K126" s="134"/>
+      <c r="L126" s="134"/>
+      <c r="M126" s="134"/>
+      <c r="N126" s="134"/>
+      <c r="O126" s="134"/>
+      <c r="P126" s="134"/>
+      <c r="Q126" s="134"/>
+      <c r="R126" s="134"/>
       <c r="S126" s="91"/>
       <c r="T126" s="108" t="s">
         <v>66</v>
@@ -9944,15 +9948,15 @@
       <c r="AB126" s="105"/>
       <c r="AC126" s="97"/>
       <c r="AD126" s="5"/>
-      <c r="AE126" s="172"/>
-      <c r="AF126" s="173"/>
-      <c r="AG126" s="173"/>
-      <c r="AH126" s="173"/>
-      <c r="AI126" s="173"/>
-      <c r="AJ126" s="135"/>
-      <c r="AK126" s="137"/>
-      <c r="AL126" s="137"/>
-      <c r="AM126" s="176"/>
+      <c r="AE126" s="171"/>
+      <c r="AF126" s="172"/>
+      <c r="AG126" s="172"/>
+      <c r="AH126" s="172"/>
+      <c r="AI126" s="172"/>
+      <c r="AJ126" s="126"/>
+      <c r="AK126" s="128"/>
+      <c r="AL126" s="128"/>
+      <c r="AM126" s="175"/>
       <c r="AN126" s="5"/>
       <c r="AO126" s="5"/>
       <c r="AP126" s="5"/>
@@ -9962,21 +9966,21 @@
       <c r="AT126" s="5"/>
     </row>
     <row r="127" spans="1:46" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="169"/>
-      <c r="B127" s="124"/>
-      <c r="C127" s="124"/>
-      <c r="D127" s="124"/>
-      <c r="E127" s="124"/>
-      <c r="F127" s="124"/>
-      <c r="G127" s="124"/>
-      <c r="H127" s="124"/>
-      <c r="I127" s="124"/>
-      <c r="J127" s="124"/>
-      <c r="K127" s="124"/>
-      <c r="L127" s="124"/>
-      <c r="M127" s="124"/>
-      <c r="N127" s="124"/>
-      <c r="O127" s="124"/>
+      <c r="A127" s="168"/>
+      <c r="B127" s="134"/>
+      <c r="C127" s="134"/>
+      <c r="D127" s="134"/>
+      <c r="E127" s="134"/>
+      <c r="F127" s="134"/>
+      <c r="G127" s="134"/>
+      <c r="H127" s="134"/>
+      <c r="I127" s="134"/>
+      <c r="J127" s="134"/>
+      <c r="K127" s="134"/>
+      <c r="L127" s="134"/>
+      <c r="M127" s="134"/>
+      <c r="N127" s="134"/>
+      <c r="O127" s="134"/>
       <c r="P127" s="103"/>
       <c r="Q127" s="103"/>
       <c r="R127" s="90"/>
@@ -9994,14 +9998,14 @@
       <c r="AB127" s="2"/>
       <c r="AC127" s="97"/>
       <c r="AD127" s="5"/>
-      <c r="AE127" s="200" t="s">
+      <c r="AE127" s="201" t="s">
         <v>68</v>
       </c>
-      <c r="AF127" s="127"/>
-      <c r="AG127" s="127"/>
-      <c r="AH127" s="127"/>
-      <c r="AI127" s="127"/>
-      <c r="AJ127" s="128"/>
+      <c r="AF127" s="136"/>
+      <c r="AG127" s="136"/>
+      <c r="AH127" s="136"/>
+      <c r="AI127" s="136"/>
+      <c r="AJ127" s="137"/>
       <c r="AK127" s="109">
         <f>AG63/AJ117</f>
         <v>0</v>
@@ -10023,25 +10027,25 @@
       <c r="AT127" s="5"/>
     </row>
     <row r="128" spans="1:46" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="203" t="s">
+      <c r="A128" s="204" t="s">
         <v>69</v>
       </c>
-      <c r="B128" s="124"/>
-      <c r="C128" s="124"/>
-      <c r="D128" s="124"/>
-      <c r="E128" s="124"/>
-      <c r="F128" s="124"/>
-      <c r="G128" s="124"/>
-      <c r="H128" s="124"/>
-      <c r="I128" s="124"/>
-      <c r="J128" s="124"/>
-      <c r="K128" s="124"/>
-      <c r="L128" s="124"/>
-      <c r="M128" s="124"/>
-      <c r="N128" s="124"/>
-      <c r="O128" s="124"/>
-      <c r="P128" s="124"/>
-      <c r="Q128" s="124"/>
+      <c r="B128" s="134"/>
+      <c r="C128" s="134"/>
+      <c r="D128" s="134"/>
+      <c r="E128" s="134"/>
+      <c r="F128" s="134"/>
+      <c r="G128" s="134"/>
+      <c r="H128" s="134"/>
+      <c r="I128" s="134"/>
+      <c r="J128" s="134"/>
+      <c r="K128" s="134"/>
+      <c r="L128" s="134"/>
+      <c r="M128" s="134"/>
+      <c r="N128" s="134"/>
+      <c r="O128" s="134"/>
+      <c r="P128" s="134"/>
+      <c r="Q128" s="134"/>
       <c r="R128" s="107"/>
       <c r="S128" s="91"/>
       <c r="T128" s="108" t="s">
@@ -10057,23 +10061,23 @@
       <c r="AB128" s="105"/>
       <c r="AC128" s="97"/>
       <c r="AD128" s="5"/>
-      <c r="AE128" s="193" t="s">
+      <c r="AE128" s="194" t="s">
         <v>71</v>
       </c>
-      <c r="AF128" s="189"/>
-      <c r="AG128" s="189"/>
-      <c r="AH128" s="189"/>
-      <c r="AI128" s="189"/>
-      <c r="AJ128" s="133"/>
-      <c r="AK128" s="204" t="e">
+      <c r="AF128" s="190"/>
+      <c r="AG128" s="190"/>
+      <c r="AH128" s="190"/>
+      <c r="AI128" s="190"/>
+      <c r="AJ128" s="124"/>
+      <c r="AK128" s="205" t="e">
         <f t="shared" ref="AK128:AM128" si="11">AK127/AK123</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AL128" s="204" t="e">
+      <c r="AL128" s="205" t="e">
         <f t="shared" si="11"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AM128" s="205" t="e">
+      <c r="AM128" s="206" t="e">
         <f t="shared" si="11"/>
         <v>#DIV/0!</v>
       </c>
@@ -10086,23 +10090,23 @@
       <c r="AT128" s="5"/>
     </row>
     <row r="129" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="124"/>
-      <c r="B129" s="124"/>
-      <c r="C129" s="124"/>
-      <c r="D129" s="124"/>
-      <c r="E129" s="124"/>
-      <c r="F129" s="124"/>
-      <c r="G129" s="124"/>
-      <c r="H129" s="124"/>
-      <c r="I129" s="124"/>
-      <c r="J129" s="124"/>
-      <c r="K129" s="124"/>
-      <c r="L129" s="124"/>
-      <c r="M129" s="124"/>
-      <c r="N129" s="124"/>
-      <c r="O129" s="124"/>
-      <c r="P129" s="124"/>
-      <c r="Q129" s="124"/>
+      <c r="A129" s="134"/>
+      <c r="B129" s="134"/>
+      <c r="C129" s="134"/>
+      <c r="D129" s="134"/>
+      <c r="E129" s="134"/>
+      <c r="F129" s="134"/>
+      <c r="G129" s="134"/>
+      <c r="H129" s="134"/>
+      <c r="I129" s="134"/>
+      <c r="J129" s="134"/>
+      <c r="K129" s="134"/>
+      <c r="L129" s="134"/>
+      <c r="M129" s="134"/>
+      <c r="N129" s="134"/>
+      <c r="O129" s="134"/>
+      <c r="P129" s="134"/>
+      <c r="Q129" s="134"/>
       <c r="R129" s="107"/>
       <c r="S129" s="91"/>
       <c r="T129" s="108" t="s">
@@ -10118,15 +10122,15 @@
       <c r="AB129" s="105"/>
       <c r="AC129" s="97"/>
       <c r="AD129" s="5"/>
-      <c r="AE129" s="172"/>
-      <c r="AF129" s="173"/>
-      <c r="AG129" s="173"/>
-      <c r="AH129" s="173"/>
-      <c r="AI129" s="173"/>
-      <c r="AJ129" s="135"/>
-      <c r="AK129" s="137"/>
-      <c r="AL129" s="137"/>
-      <c r="AM129" s="176"/>
+      <c r="AE129" s="171"/>
+      <c r="AF129" s="172"/>
+      <c r="AG129" s="172"/>
+      <c r="AH129" s="172"/>
+      <c r="AI129" s="172"/>
+      <c r="AJ129" s="126"/>
+      <c r="AK129" s="128"/>
+      <c r="AL129" s="128"/>
+      <c r="AM129" s="175"/>
       <c r="AN129" s="5"/>
       <c r="AO129" s="5"/>
       <c r="AP129" s="5"/>
@@ -10136,26 +10140,26 @@
       <c r="AT129" s="5"/>
     </row>
     <row r="130" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="206" t="s">
+      <c r="A130" s="207" t="s">
         <v>73</v>
       </c>
-      <c r="B130" s="124"/>
-      <c r="C130" s="124"/>
-      <c r="D130" s="124"/>
-      <c r="E130" s="124"/>
-      <c r="F130" s="124"/>
-      <c r="G130" s="124"/>
-      <c r="H130" s="124"/>
-      <c r="I130" s="124"/>
-      <c r="J130" s="124"/>
-      <c r="K130" s="124"/>
-      <c r="L130" s="124"/>
-      <c r="M130" s="124"/>
-      <c r="N130" s="124"/>
-      <c r="O130" s="124"/>
-      <c r="P130" s="124"/>
-      <c r="Q130" s="124"/>
-      <c r="R130" s="124"/>
+      <c r="B130" s="134"/>
+      <c r="C130" s="134"/>
+      <c r="D130" s="134"/>
+      <c r="E130" s="134"/>
+      <c r="F130" s="134"/>
+      <c r="G130" s="134"/>
+      <c r="H130" s="134"/>
+      <c r="I130" s="134"/>
+      <c r="J130" s="134"/>
+      <c r="K130" s="134"/>
+      <c r="L130" s="134"/>
+      <c r="M130" s="134"/>
+      <c r="N130" s="134"/>
+      <c r="O130" s="134"/>
+      <c r="P130" s="134"/>
+      <c r="Q130" s="134"/>
+      <c r="R130" s="134"/>
       <c r="S130" s="91"/>
       <c r="T130" s="108" t="s">
         <v>74</v>
@@ -10170,21 +10174,21 @@
       <c r="AB130" s="105"/>
       <c r="AC130" s="97"/>
       <c r="AD130" s="112"/>
-      <c r="AE130" s="193" t="s">
+      <c r="AE130" s="194" t="s">
         <v>75</v>
       </c>
-      <c r="AF130" s="189"/>
-      <c r="AG130" s="189"/>
-      <c r="AH130" s="189"/>
-      <c r="AI130" s="189"/>
-      <c r="AJ130" s="133"/>
-      <c r="AK130" s="136">
+      <c r="AF130" s="190"/>
+      <c r="AG130" s="190"/>
+      <c r="AH130" s="190"/>
+      <c r="AI130" s="190"/>
+      <c r="AJ130" s="124"/>
+      <c r="AK130" s="127">
         <v>0</v>
       </c>
-      <c r="AL130" s="136">
+      <c r="AL130" s="127">
         <v>0</v>
       </c>
-      <c r="AM130" s="207">
+      <c r="AM130" s="208">
         <f>AK130+AL130</f>
         <v>0</v>
       </c>
@@ -10197,24 +10201,24 @@
       <c r="AT130" s="5"/>
     </row>
     <row r="131" spans="1:46" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="124"/>
-      <c r="B131" s="124"/>
-      <c r="C131" s="124"/>
-      <c r="D131" s="124"/>
-      <c r="E131" s="124"/>
-      <c r="F131" s="124"/>
-      <c r="G131" s="124"/>
-      <c r="H131" s="124"/>
-      <c r="I131" s="124"/>
-      <c r="J131" s="124"/>
-      <c r="K131" s="124"/>
-      <c r="L131" s="124"/>
-      <c r="M131" s="124"/>
-      <c r="N131" s="124"/>
-      <c r="O131" s="124"/>
-      <c r="P131" s="124"/>
-      <c r="Q131" s="124"/>
-      <c r="R131" s="124"/>
+      <c r="A131" s="134"/>
+      <c r="B131" s="134"/>
+      <c r="C131" s="134"/>
+      <c r="D131" s="134"/>
+      <c r="E131" s="134"/>
+      <c r="F131" s="134"/>
+      <c r="G131" s="134"/>
+      <c r="H131" s="134"/>
+      <c r="I131" s="134"/>
+      <c r="J131" s="134"/>
+      <c r="K131" s="134"/>
+      <c r="L131" s="134"/>
+      <c r="M131" s="134"/>
+      <c r="N131" s="134"/>
+      <c r="O131" s="134"/>
+      <c r="P131" s="134"/>
+      <c r="Q131" s="134"/>
+      <c r="R131" s="134"/>
       <c r="S131" s="91"/>
       <c r="T131" s="108" t="s">
         <v>76</v>
@@ -10229,15 +10233,15 @@
       <c r="AB131" s="2"/>
       <c r="AC131" s="97"/>
       <c r="AD131" s="5"/>
-      <c r="AE131" s="172"/>
-      <c r="AF131" s="173"/>
-      <c r="AG131" s="173"/>
-      <c r="AH131" s="173"/>
-      <c r="AI131" s="173"/>
-      <c r="AJ131" s="135"/>
-      <c r="AK131" s="137"/>
-      <c r="AL131" s="137"/>
-      <c r="AM131" s="176"/>
+      <c r="AE131" s="171"/>
+      <c r="AF131" s="172"/>
+      <c r="AG131" s="172"/>
+      <c r="AH131" s="172"/>
+      <c r="AI131" s="172"/>
+      <c r="AJ131" s="126"/>
+      <c r="AK131" s="128"/>
+      <c r="AL131" s="128"/>
+      <c r="AM131" s="175"/>
       <c r="AN131" s="5"/>
       <c r="AO131" s="5"/>
       <c r="AP131" s="5"/>
@@ -10281,23 +10285,23 @@
       <c r="AB132" s="105"/>
       <c r="AC132" s="97"/>
       <c r="AD132" s="5"/>
-      <c r="AE132" s="208" t="s">
+      <c r="AE132" s="209" t="s">
         <v>79</v>
       </c>
-      <c r="AF132" s="189"/>
-      <c r="AG132" s="189"/>
-      <c r="AH132" s="189"/>
-      <c r="AI132" s="189"/>
-      <c r="AJ132" s="133"/>
-      <c r="AK132" s="209">
+      <c r="AF132" s="190"/>
+      <c r="AG132" s="190"/>
+      <c r="AH132" s="190"/>
+      <c r="AI132" s="190"/>
+      <c r="AJ132" s="124"/>
+      <c r="AK132" s="210">
         <f>COUNTIF(AH13:AI62,"NLS")</f>
         <v>0</v>
       </c>
-      <c r="AL132" s="209">
+      <c r="AL132" s="210">
         <f>COUNTIF(AH64:AI113,"NLS")</f>
         <v>0</v>
       </c>
-      <c r="AM132" s="187">
+      <c r="AM132" s="188">
         <f>AK132+AL132</f>
         <v>0</v>
       </c>
@@ -10313,24 +10317,24 @@
       <c r="A133" s="101" t="s">
         <v>80</v>
       </c>
-      <c r="B133" s="206" t="s">
+      <c r="B133" s="207" t="s">
         <v>81</v>
       </c>
-      <c r="C133" s="124"/>
-      <c r="D133" s="124"/>
-      <c r="E133" s="124"/>
-      <c r="F133" s="124"/>
-      <c r="G133" s="124"/>
-      <c r="H133" s="124"/>
-      <c r="I133" s="124"/>
-      <c r="J133" s="124"/>
-      <c r="K133" s="124"/>
-      <c r="L133" s="124"/>
-      <c r="M133" s="124"/>
-      <c r="N133" s="124"/>
-      <c r="O133" s="124"/>
-      <c r="P133" s="124"/>
-      <c r="Q133" s="124"/>
+      <c r="C133" s="134"/>
+      <c r="D133" s="134"/>
+      <c r="E133" s="134"/>
+      <c r="F133" s="134"/>
+      <c r="G133" s="134"/>
+      <c r="H133" s="134"/>
+      <c r="I133" s="134"/>
+      <c r="J133" s="134"/>
+      <c r="K133" s="134"/>
+      <c r="L133" s="134"/>
+      <c r="M133" s="134"/>
+      <c r="N133" s="134"/>
+      <c r="O133" s="134"/>
+      <c r="P133" s="134"/>
+      <c r="Q133" s="134"/>
       <c r="R133" s="90"/>
       <c r="S133" s="91"/>
       <c r="T133" s="108" t="s">
@@ -10346,15 +10350,15 @@
       <c r="AB133" s="2"/>
       <c r="AC133" s="97"/>
       <c r="AD133" s="5"/>
-      <c r="AE133" s="172"/>
-      <c r="AF133" s="173"/>
-      <c r="AG133" s="173"/>
-      <c r="AH133" s="173"/>
-      <c r="AI133" s="173"/>
-      <c r="AJ133" s="135"/>
-      <c r="AK133" s="137"/>
-      <c r="AL133" s="137"/>
-      <c r="AM133" s="176"/>
+      <c r="AE133" s="171"/>
+      <c r="AF133" s="172"/>
+      <c r="AG133" s="172"/>
+      <c r="AH133" s="172"/>
+      <c r="AI133" s="172"/>
+      <c r="AJ133" s="126"/>
+      <c r="AK133" s="128"/>
+      <c r="AL133" s="128"/>
+      <c r="AM133" s="175"/>
       <c r="AN133" s="5"/>
       <c r="AO133" s="5"/>
       <c r="AP133" s="5"/>
@@ -10396,23 +10400,23 @@
       <c r="AB134" s="5"/>
       <c r="AC134" s="97"/>
       <c r="AD134" s="5"/>
-      <c r="AE134" s="208" t="s">
+      <c r="AE134" s="209" t="s">
         <v>84</v>
       </c>
-      <c r="AF134" s="189"/>
-      <c r="AG134" s="189"/>
-      <c r="AH134" s="189"/>
-      <c r="AI134" s="189"/>
-      <c r="AJ134" s="133"/>
-      <c r="AK134" s="210">
+      <c r="AF134" s="190"/>
+      <c r="AG134" s="190"/>
+      <c r="AH134" s="190"/>
+      <c r="AI134" s="190"/>
+      <c r="AJ134" s="124"/>
+      <c r="AK134" s="211">
         <f>COUNTIF(AH13:AI62,"Transferred Out")</f>
         <v>0</v>
       </c>
-      <c r="AL134" s="210">
+      <c r="AL134" s="211">
         <f>COUNTIF(AH64:AI113,"Transferred Out")</f>
         <v>0</v>
       </c>
-      <c r="AM134" s="207">
+      <c r="AM134" s="208">
         <f>AK134+AL134</f>
         <v>0</v>
       </c>
@@ -10457,15 +10461,15 @@
       <c r="AB135" s="105"/>
       <c r="AC135" s="97"/>
       <c r="AD135" s="5"/>
-      <c r="AE135" s="172"/>
-      <c r="AF135" s="173"/>
-      <c r="AG135" s="173"/>
-      <c r="AH135" s="173"/>
-      <c r="AI135" s="173"/>
-      <c r="AJ135" s="135"/>
-      <c r="AK135" s="137"/>
-      <c r="AL135" s="137"/>
-      <c r="AM135" s="176"/>
+      <c r="AE135" s="171"/>
+      <c r="AF135" s="172"/>
+      <c r="AG135" s="172"/>
+      <c r="AH135" s="172"/>
+      <c r="AI135" s="172"/>
+      <c r="AJ135" s="126"/>
+      <c r="AK135" s="128"/>
+      <c r="AL135" s="128"/>
+      <c r="AM135" s="175"/>
       <c r="AN135" s="5"/>
       <c r="AO135" s="5"/>
       <c r="AP135" s="5"/>
@@ -10476,15 +10480,15 @@
     </row>
     <row r="136" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="5"/>
-      <c r="B136" s="215"/>
-      <c r="C136" s="124"/>
-      <c r="D136" s="124"/>
-      <c r="E136" s="124"/>
-      <c r="F136" s="124"/>
-      <c r="G136" s="124"/>
-      <c r="H136" s="124"/>
-      <c r="I136" s="124"/>
-      <c r="J136" s="124"/>
+      <c r="B136" s="216"/>
+      <c r="C136" s="134"/>
+      <c r="D136" s="134"/>
+      <c r="E136" s="134"/>
+      <c r="F136" s="134"/>
+      <c r="G136" s="134"/>
+      <c r="H136" s="134"/>
+      <c r="I136" s="134"/>
+      <c r="J136" s="134"/>
       <c r="K136" s="5"/>
       <c r="L136" s="5"/>
       <c r="M136" s="5"/>
@@ -10507,23 +10511,23 @@
       <c r="AB136" s="5"/>
       <c r="AC136" s="97"/>
       <c r="AD136" s="115"/>
-      <c r="AE136" s="208" t="s">
+      <c r="AE136" s="209" t="s">
         <v>87</v>
       </c>
-      <c r="AF136" s="189"/>
-      <c r="AG136" s="189"/>
-      <c r="AH136" s="189"/>
-      <c r="AI136" s="189"/>
-      <c r="AJ136" s="133"/>
-      <c r="AK136" s="210">
+      <c r="AF136" s="190"/>
+      <c r="AG136" s="190"/>
+      <c r="AH136" s="190"/>
+      <c r="AI136" s="190"/>
+      <c r="AJ136" s="124"/>
+      <c r="AK136" s="211">
         <f>COUNTIF(AH13:AI62,"Transferred In")</f>
         <v>0</v>
       </c>
-      <c r="AL136" s="210">
+      <c r="AL136" s="211">
         <f>COUNTIF(AH64:AI113,"Transferred In")</f>
         <v>0</v>
       </c>
-      <c r="AM136" s="207">
+      <c r="AM136" s="208">
         <f>AK136+AL136</f>
         <v>0</v>
       </c>
@@ -10537,15 +10541,15 @@
     </row>
     <row r="137" spans="1:46" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A137" s="5"/>
-      <c r="B137" s="124"/>
-      <c r="C137" s="124"/>
-      <c r="D137" s="124"/>
-      <c r="E137" s="124"/>
-      <c r="F137" s="124"/>
-      <c r="G137" s="124"/>
-      <c r="H137" s="124"/>
-      <c r="I137" s="124"/>
-      <c r="J137" s="124"/>
+      <c r="B137" s="134"/>
+      <c r="C137" s="134"/>
+      <c r="D137" s="134"/>
+      <c r="E137" s="134"/>
+      <c r="F137" s="134"/>
+      <c r="G137" s="134"/>
+      <c r="H137" s="134"/>
+      <c r="I137" s="134"/>
+      <c r="J137" s="134"/>
       <c r="K137" s="5"/>
       <c r="L137" s="5"/>
       <c r="M137" s="5"/>
@@ -10568,15 +10572,15 @@
       <c r="AB137" s="5"/>
       <c r="AC137" s="97"/>
       <c r="AD137" s="5"/>
-      <c r="AE137" s="162"/>
-      <c r="AF137" s="158"/>
-      <c r="AG137" s="158"/>
-      <c r="AH137" s="158"/>
-      <c r="AI137" s="158"/>
-      <c r="AJ137" s="216"/>
-      <c r="AK137" s="217"/>
-      <c r="AL137" s="217"/>
-      <c r="AM137" s="218"/>
+      <c r="AE137" s="152"/>
+      <c r="AF137" s="148"/>
+      <c r="AG137" s="148"/>
+      <c r="AH137" s="148"/>
+      <c r="AI137" s="148"/>
+      <c r="AJ137" s="217"/>
+      <c r="AK137" s="218"/>
+      <c r="AL137" s="218"/>
+      <c r="AM137" s="219"/>
       <c r="AN137" s="5"/>
       <c r="AO137" s="5"/>
       <c r="AP137" s="5"/>
@@ -10720,15 +10724,15 @@
       <c r="AB140" s="5"/>
       <c r="AC140" s="97"/>
       <c r="AD140" s="5"/>
-      <c r="AE140" s="142"/>
-      <c r="AF140" s="219"/>
-      <c r="AG140" s="219"/>
-      <c r="AH140" s="219"/>
-      <c r="AI140" s="219"/>
-      <c r="AJ140" s="219"/>
-      <c r="AK140" s="219"/>
-      <c r="AL140" s="219"/>
-      <c r="AM140" s="219"/>
+      <c r="AE140" s="133"/>
+      <c r="AF140" s="220"/>
+      <c r="AG140" s="220"/>
+      <c r="AH140" s="220"/>
+      <c r="AI140" s="220"/>
+      <c r="AJ140" s="220"/>
+      <c r="AK140" s="220"/>
+      <c r="AL140" s="220"/>
+      <c r="AM140" s="220"/>
       <c r="AN140" s="5"/>
       <c r="AO140" s="5"/>
       <c r="AP140" s="5"/>
@@ -10757,28 +10761,28 @@
       <c r="Q141" s="5"/>
       <c r="R141" s="5"/>
       <c r="S141" s="91"/>
-      <c r="T141" s="220" t="s">
+      <c r="T141" s="221" t="s">
         <v>93</v>
       </c>
-      <c r="U141" s="124"/>
-      <c r="V141" s="124"/>
-      <c r="W141" s="124"/>
-      <c r="X141" s="124"/>
-      <c r="Y141" s="124"/>
-      <c r="Z141" s="124"/>
-      <c r="AA141" s="124"/>
-      <c r="AB141" s="124"/>
-      <c r="AC141" s="161"/>
+      <c r="U141" s="134"/>
+      <c r="V141" s="134"/>
+      <c r="W141" s="134"/>
+      <c r="X141" s="134"/>
+      <c r="Y141" s="134"/>
+      <c r="Z141" s="134"/>
+      <c r="AA141" s="134"/>
+      <c r="AB141" s="134"/>
+      <c r="AC141" s="151"/>
       <c r="AD141" s="5"/>
-      <c r="AE141" s="213"/>
-      <c r="AF141" s="213"/>
-      <c r="AG141" s="213"/>
-      <c r="AH141" s="213"/>
-      <c r="AI141" s="213"/>
-      <c r="AJ141" s="213"/>
-      <c r="AK141" s="213"/>
-      <c r="AL141" s="213"/>
-      <c r="AM141" s="213"/>
+      <c r="AE141" s="214"/>
+      <c r="AF141" s="214"/>
+      <c r="AG141" s="214"/>
+      <c r="AH141" s="214"/>
+      <c r="AI141" s="214"/>
+      <c r="AJ141" s="214"/>
+      <c r="AK141" s="214"/>
+      <c r="AL141" s="214"/>
+      <c r="AM141" s="214"/>
       <c r="AN141" s="5"/>
       <c r="AO141" s="5"/>
       <c r="AP141" s="5"/>
@@ -10807,28 +10811,28 @@
       <c r="Q142" s="5"/>
       <c r="R142" s="5"/>
       <c r="S142" s="91"/>
-      <c r="T142" s="153"/>
-      <c r="U142" s="124"/>
-      <c r="V142" s="124"/>
-      <c r="W142" s="124"/>
-      <c r="X142" s="124"/>
-      <c r="Y142" s="124"/>
-      <c r="Z142" s="124"/>
-      <c r="AA142" s="124"/>
-      <c r="AB142" s="124"/>
-      <c r="AC142" s="161"/>
+      <c r="T142" s="143"/>
+      <c r="U142" s="134"/>
+      <c r="V142" s="134"/>
+      <c r="W142" s="134"/>
+      <c r="X142" s="134"/>
+      <c r="Y142" s="134"/>
+      <c r="Z142" s="134"/>
+      <c r="AA142" s="134"/>
+      <c r="AB142" s="134"/>
+      <c r="AC142" s="151"/>
       <c r="AD142" s="5"/>
-      <c r="AE142" s="214" t="s">
+      <c r="AE142" s="215" t="s">
         <v>94</v>
       </c>
-      <c r="AF142" s="189"/>
-      <c r="AG142" s="189"/>
-      <c r="AH142" s="189"/>
-      <c r="AI142" s="189"/>
-      <c r="AJ142" s="189"/>
-      <c r="AK142" s="189"/>
-      <c r="AL142" s="189"/>
-      <c r="AM142" s="189"/>
+      <c r="AF142" s="190"/>
+      <c r="AG142" s="190"/>
+      <c r="AH142" s="190"/>
+      <c r="AI142" s="190"/>
+      <c r="AJ142" s="190"/>
+      <c r="AK142" s="190"/>
+      <c r="AL142" s="190"/>
+      <c r="AM142" s="190"/>
       <c r="AN142" s="5"/>
       <c r="AO142" s="5"/>
       <c r="AP142" s="5"/>
@@ -10940,8 +10944,8 @@
       <c r="AT144" s="5"/>
     </row>
     <row r="145" spans="1:46" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A145" s="211"/>
-      <c r="B145" s="124"/>
+      <c r="A145" s="212"/>
+      <c r="B145" s="134"/>
       <c r="C145" s="119"/>
       <c r="D145" s="119"/>
       <c r="E145" s="119"/>
@@ -10972,15 +10976,15 @@
       <c r="AB145" s="5"/>
       <c r="AC145" s="118"/>
       <c r="AD145" s="5"/>
-      <c r="AE145" s="212"/>
-      <c r="AF145" s="213"/>
-      <c r="AG145" s="213"/>
-      <c r="AH145" s="213"/>
-      <c r="AI145" s="213"/>
-      <c r="AJ145" s="213"/>
-      <c r="AK145" s="213"/>
-      <c r="AL145" s="213"/>
-      <c r="AM145" s="213"/>
+      <c r="AE145" s="213"/>
+      <c r="AF145" s="214"/>
+      <c r="AG145" s="214"/>
+      <c r="AH145" s="214"/>
+      <c r="AI145" s="214"/>
+      <c r="AJ145" s="214"/>
+      <c r="AK145" s="214"/>
+      <c r="AL145" s="214"/>
+      <c r="AM145" s="214"/>
       <c r="AN145" s="5"/>
       <c r="AO145" s="5"/>
       <c r="AP145" s="5"/>
@@ -10990,8 +10994,8 @@
       <c r="AT145" s="5"/>
     </row>
     <row r="146" spans="1:46" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A146" s="124"/>
-      <c r="B146" s="124"/>
+      <c r="A146" s="134"/>
+      <c r="B146" s="134"/>
       <c r="C146" s="119"/>
       <c r="D146" s="119"/>
       <c r="E146" s="119"/>
@@ -11022,17 +11026,17 @@
       <c r="AB146" s="121"/>
       <c r="AC146" s="122"/>
       <c r="AD146" s="5"/>
-      <c r="AE146" s="214" t="s">
+      <c r="AE146" s="215" t="s">
         <v>100</v>
       </c>
-      <c r="AF146" s="189"/>
-      <c r="AG146" s="189"/>
-      <c r="AH146" s="189"/>
-      <c r="AI146" s="189"/>
-      <c r="AJ146" s="189"/>
-      <c r="AK146" s="189"/>
-      <c r="AL146" s="189"/>
-      <c r="AM146" s="189"/>
+      <c r="AF146" s="190"/>
+      <c r="AG146" s="190"/>
+      <c r="AH146" s="190"/>
+      <c r="AI146" s="190"/>
+      <c r="AJ146" s="190"/>
+      <c r="AK146" s="190"/>
+      <c r="AL146" s="190"/>
+      <c r="AM146" s="190"/>
       <c r="AN146" s="5"/>
       <c r="AO146" s="5"/>
       <c r="AP146" s="5"/>
@@ -21545,8 +21549,8 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.17" right="0.16" top="0.18" bottom="0.19" header="0" footer="0"/>
-  <pageSetup scale="62" orientation="landscape"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup paperSize="10000" scale="62" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>